<commit_message>
🔄 Auto-collect traffic data: 2026-10-19 10:32 AM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-10-19_Mon.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-10-19_Mon.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="All Periods Combined" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="359">
   <si>
     <t>Date</t>
   </si>
@@ -122,7 +123,7 @@
     <t>12:00 AM</t>
   </si>
   <si>
-    <t>Sunday (Weekend) - Night Off-Peak</t>
+    <t>Monday (Weekday) - Night Off-Peak</t>
   </si>
   <si>
     <t>Blue Line</t>
@@ -716,6 +717,327 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/12_00_AM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>10/19/2026, 10:03:28 AM</t>
+  </si>
+  <si>
+    <t>10:00 AM</t>
+  </si>
+  <si>
+    <t>Monday (Weekday) - Morning Peak</t>
+  </si>
+  <si>
+    <t> | 30 min | 1:00 PM—1:30 PM | Blue Line</t>
+  </si>
+  <si>
+    <t> | 35 min | 12.2 km | via Barrackpore Trunk Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>5 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.17x</t>
+  </si>
+  <si>
+    <t>14.3% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:03:48 AM</t>
+  </si>
+  <si>
+    <t> | 33 min | 1:00 PM—1:33 PM | Blue Line | 1:00 PM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 47 min | 15.8 km | via Netaji Subhas Chandra Bose Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.42x</t>
+  </si>
+  <si>
+    <t>29.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:05:28 AM</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:07:10 AM</t>
+  </si>
+  <si>
+    <t> | 18 min | 5.2 km | via Jatindra Mohan Ave and Central Ave/Chittaranjan Ave | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:08:53 AM</t>
+  </si>
+  <si>
+    <t> | 16 min | 5.6 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:09:11 AM</t>
+  </si>
+  <si>
+    <t> | 14 min | 1:00 PM—1:14 PM | Blue Line</t>
+  </si>
+  <si>
+    <t> | 18 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>4 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.29x</t>
+  </si>
+  <si>
+    <t>22.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:10:53 AM</t>
+  </si>
+  <si>
+    <t> | 24 min | 7.8 km | via Chowringee Rd/Jawaharlal Nehru Rd and Ashutosh Mukherjee Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:11:12 AM</t>
+  </si>
+  <si>
+    <t> | 17 min | 12:54 PM—1:11 PM | Blue Line</t>
+  </si>
+  <si>
+    <t> | 20 min | 6.4 km | via Netaji Subhas Chandra Bose Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>3 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.18x</t>
+  </si>
+  <si>
+    <t>15.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:11:30 AM</t>
+  </si>
+  <si>
+    <t> | 16 min | 1:00 PM—1:16 PM | Blue Line</t>
+  </si>
+  <si>
+    <t> | 29 min | 8.6 km | via Jessore Rd and Lock Gate Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.81x</t>
+  </si>
+  <si>
+    <t>44.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:11:49 AM</t>
+  </si>
+  <si>
+    <t> | 30 min | 1:32 PM—2:02 PM | Green Line | 1:32 PM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 35 min | 10.8 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:13:32 AM</t>
+  </si>
+  <si>
+    <t> | 21 min | 8.0 km | via Beleghata Main Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:15:17 AM</t>
+  </si>
+  <si>
+    <t> | 28 min | 6.8 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:16:59 AM</t>
+  </si>
+  <si>
+    <t> | 16 min | 4.9 km | via Narkeldanga Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:17:18 AM</t>
+  </si>
+  <si>
+    <t> | 12 min | 1:32 PM—1:44 PM | Green Line</t>
+  </si>
+  <si>
+    <t> | 27 min | 7.6 km | via Kali Krishna Tagore St | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>15 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.25x</t>
+  </si>
+  <si>
+    <t>55.6% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:17:36 AM</t>
+  </si>
+  <si>
+    <t> | 25 min | 1:37 PM—2:02 PM | Green Line</t>
+  </si>
+  <si>
+    <t> | 28 min | 15.7 km | via Circus Ave | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.12x</t>
+  </si>
+  <si>
+    <t>10.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:19:18 AM</t>
+  </si>
+  <si>
+    <t> | 20 min | 9.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:20:57 AM</t>
+  </si>
+  <si>
+    <t> | 8 min | 4.4 km | via Bangaon - Kulpi Rd/Biswa Bangla Sarani/Eastern Metropolitan Bypass/Thakurnagar - Panchpota Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:22:39 AM</t>
+  </si>
+  <si>
+    <t> | 17 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:24:20 AM</t>
+  </si>
+  <si>
+    <t> | 21 min | 7.8 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:26:00 AM</t>
+  </si>
+  <si>
+    <t> | 10 min | 3.7 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:27:40 AM</t>
+  </si>
+  <si>
+    <t> | 11 min | 4.1 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:29:23 AM</t>
+  </si>
+  <si>
+    <t> | 19 min | 6.5 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:31:06 AM</t>
+  </si>
+  <si>
+    <t> | 8 min | 2.4 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 10:32:49 AM</t>
+  </si>
+  <si>
+    <t> | 3 min | 1.3 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -741,6 +1063,33 @@
   </si>
   <si>
     <t>12:00 AM Savings (%)</t>
+  </si>
+  <si>
+    <t>10:00 AM Scraped At</t>
+  </si>
+  <si>
+    <t>10:00 AM Actual Metro</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Walk</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Route</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>10:00 AM Car (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Faster Mode</t>
+  </si>
+  <si>
+    <t>10:00 AM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -3276,10 +3625,2131 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>13.4</v>
+      </c>
+      <c r="J2">
+        <v>12.2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>235</v>
+      </c>
+      <c r="L2" t="s">
+        <v>236</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2">
+        <v>30</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>237</v>
+      </c>
+      <c r="R2">
+        <v>35</v>
+      </c>
+      <c r="S2" t="s">
+        <v>238</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="U2" t="s">
+        <v>240</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" t="s">
+        <v>241</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>242</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>244</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.5</v>
+      </c>
+      <c r="J3">
+        <v>15.8</v>
+      </c>
+      <c r="K3" t="s">
+        <v>235</v>
+      </c>
+      <c r="L3" t="s">
+        <v>236</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3">
+        <v>33</v>
+      </c>
+      <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>245</v>
+      </c>
+      <c r="R3">
+        <v>47</v>
+      </c>
+      <c r="S3" t="s">
+        <v>246</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" t="s">
+        <v>247</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>248</v>
+      </c>
+      <c r="X3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>249</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>251</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>3.8</v>
+      </c>
+      <c r="J4">
+        <v>4.1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>235</v>
+      </c>
+      <c r="L4" t="s">
+        <v>236</v>
+      </c>
+      <c r="M4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" t="s">
+        <v>187</v>
+      </c>
+      <c r="P4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R4">
+        <v>16</v>
+      </c>
+      <c r="S4" t="s">
+        <v>64</v>
+      </c>
+      <c r="T4" t="s">
+        <v>38</v>
+      </c>
+      <c r="U4" t="s">
+        <v>38</v>
+      </c>
+      <c r="V4" t="s">
+        <v>38</v>
+      </c>
+      <c r="W4" t="s">
+        <v>38</v>
+      </c>
+      <c r="X4" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>253</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>5.2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>235</v>
+      </c>
+      <c r="L5" t="s">
+        <v>236</v>
+      </c>
+      <c r="M5" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" t="s">
+        <v>187</v>
+      </c>
+      <c r="P5" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>38</v>
+      </c>
+      <c r="R5">
+        <v>18</v>
+      </c>
+      <c r="S5" t="s">
+        <v>254</v>
+      </c>
+      <c r="T5" t="s">
+        <v>38</v>
+      </c>
+      <c r="U5" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" t="s">
+        <v>38</v>
+      </c>
+      <c r="W5" t="s">
+        <v>38</v>
+      </c>
+      <c r="X5" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>256</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.6</v>
+      </c>
+      <c r="K6" t="s">
+        <v>235</v>
+      </c>
+      <c r="L6" t="s">
+        <v>236</v>
+      </c>
+      <c r="M6" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" t="s">
+        <v>187</v>
+      </c>
+      <c r="P6" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>38</v>
+      </c>
+      <c r="R6">
+        <v>16</v>
+      </c>
+      <c r="S6" t="s">
+        <v>257</v>
+      </c>
+      <c r="T6" t="s">
+        <v>38</v>
+      </c>
+      <c r="U6" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6" t="s">
+        <v>38</v>
+      </c>
+      <c r="W6" t="s">
+        <v>38</v>
+      </c>
+      <c r="X6" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>7.7</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>235</v>
+      </c>
+      <c r="L7" t="s">
+        <v>236</v>
+      </c>
+      <c r="M7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>14</v>
+      </c>
+      <c r="P7" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>260</v>
+      </c>
+      <c r="R7">
+        <v>18</v>
+      </c>
+      <c r="S7" t="s">
+        <v>261</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="U7" t="s">
+        <v>263</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>264</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>265</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>267</v>
+      </c>
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>99</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>7.8</v>
+      </c>
+      <c r="K8" t="s">
+        <v>235</v>
+      </c>
+      <c r="L8" t="s">
+        <v>236</v>
+      </c>
+      <c r="M8" t="s">
+        <v>38</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8" t="s">
+        <v>187</v>
+      </c>
+      <c r="P8" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>38</v>
+      </c>
+      <c r="R8">
+        <v>24</v>
+      </c>
+      <c r="S8" t="s">
+        <v>268</v>
+      </c>
+      <c r="T8" t="s">
+        <v>38</v>
+      </c>
+      <c r="U8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V8" t="s">
+        <v>38</v>
+      </c>
+      <c r="W8" t="s">
+        <v>38</v>
+      </c>
+      <c r="X8" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>270</v>
+      </c>
+      <c r="D9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>99</v>
+      </c>
+      <c r="H9" t="s">
+        <v>109</v>
+      </c>
+      <c r="I9">
+        <v>7</v>
+      </c>
+      <c r="J9">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="s">
+        <v>235</v>
+      </c>
+      <c r="L9" t="s">
+        <v>236</v>
+      </c>
+      <c r="M9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9">
+        <v>17</v>
+      </c>
+      <c r="P9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>271</v>
+      </c>
+      <c r="R9">
+        <v>20</v>
+      </c>
+      <c r="S9" t="s">
+        <v>272</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="U9" t="s">
+        <v>274</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W9" t="s">
+        <v>275</v>
+      </c>
+      <c r="X9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>276</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>9.8</v>
+      </c>
+      <c r="J10">
+        <v>8.6</v>
+      </c>
+      <c r="K10" t="s">
+        <v>235</v>
+      </c>
+      <c r="L10" t="s">
+        <v>236</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10">
+        <v>16</v>
+      </c>
+      <c r="P10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>279</v>
+      </c>
+      <c r="R10">
+        <v>29</v>
+      </c>
+      <c r="S10" t="s">
+        <v>280</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="U10" t="s">
+        <v>281</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W10" t="s">
+        <v>282</v>
+      </c>
+      <c r="X10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>283</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>285</v>
+      </c>
+      <c r="D11" t="s">
+        <v>127</v>
+      </c>
+      <c r="E11" t="s">
+        <v>128</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" t="s">
+        <v>130</v>
+      </c>
+      <c r="I11">
+        <v>13.4</v>
+      </c>
+      <c r="J11">
+        <v>10.8</v>
+      </c>
+      <c r="K11" t="s">
+        <v>235</v>
+      </c>
+      <c r="L11" t="s">
+        <v>236</v>
+      </c>
+      <c r="M11" t="s">
+        <v>131</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11">
+        <v>30</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>286</v>
+      </c>
+      <c r="R11">
+        <v>35</v>
+      </c>
+      <c r="S11" t="s">
+        <v>287</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="U11" t="s">
+        <v>240</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W11" t="s">
+        <v>241</v>
+      </c>
+      <c r="X11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>288</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>290</v>
+      </c>
+      <c r="D12" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" t="s">
+        <v>128</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>140</v>
+      </c>
+      <c r="H12" t="s">
+        <v>130</v>
+      </c>
+      <c r="I12">
+        <v>8.6</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>235</v>
+      </c>
+      <c r="L12" t="s">
+        <v>236</v>
+      </c>
+      <c r="M12" t="s">
+        <v>38</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12" t="s">
+        <v>187</v>
+      </c>
+      <c r="P12" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>38</v>
+      </c>
+      <c r="R12">
+        <v>21</v>
+      </c>
+      <c r="S12" t="s">
+        <v>291</v>
+      </c>
+      <c r="T12" t="s">
+        <v>38</v>
+      </c>
+      <c r="U12" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12" t="s">
+        <v>38</v>
+      </c>
+      <c r="W12" t="s">
+        <v>38</v>
+      </c>
+      <c r="X12" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>293</v>
+      </c>
+      <c r="D13" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" t="s">
+        <v>128</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" t="s">
+        <v>140</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>6.8</v>
+      </c>
+      <c r="K13" t="s">
+        <v>235</v>
+      </c>
+      <c r="L13" t="s">
+        <v>236</v>
+      </c>
+      <c r="M13" t="s">
+        <v>38</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13" t="s">
+        <v>187</v>
+      </c>
+      <c r="P13" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>38</v>
+      </c>
+      <c r="R13">
+        <v>28</v>
+      </c>
+      <c r="S13" t="s">
+        <v>294</v>
+      </c>
+      <c r="T13" t="s">
+        <v>38</v>
+      </c>
+      <c r="U13" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13" t="s">
+        <v>38</v>
+      </c>
+      <c r="W13" t="s">
+        <v>38</v>
+      </c>
+      <c r="X13" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>296</v>
+      </c>
+      <c r="D14" t="s">
+        <v>157</v>
+      </c>
+      <c r="E14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>158</v>
+      </c>
+      <c r="H14" t="s">
+        <v>130</v>
+      </c>
+      <c r="I14">
+        <v>6.6</v>
+      </c>
+      <c r="J14">
+        <v>4.9</v>
+      </c>
+      <c r="K14" t="s">
+        <v>235</v>
+      </c>
+      <c r="L14" t="s">
+        <v>236</v>
+      </c>
+      <c r="M14" t="s">
+        <v>38</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14" t="s">
+        <v>187</v>
+      </c>
+      <c r="P14" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>38</v>
+      </c>
+      <c r="R14">
+        <v>16</v>
+      </c>
+      <c r="S14" t="s">
+        <v>297</v>
+      </c>
+      <c r="T14" t="s">
+        <v>38</v>
+      </c>
+      <c r="U14" t="s">
+        <v>38</v>
+      </c>
+      <c r="V14" t="s">
+        <v>38</v>
+      </c>
+      <c r="W14" t="s">
+        <v>38</v>
+      </c>
+      <c r="X14" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>299</v>
+      </c>
+      <c r="D15" t="s">
+        <v>168</v>
+      </c>
+      <c r="E15" t="s">
+        <v>128</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" t="s">
+        <v>158</v>
+      </c>
+      <c r="I15">
+        <v>7.3</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>235</v>
+      </c>
+      <c r="L15" t="s">
+        <v>236</v>
+      </c>
+      <c r="M15" t="s">
+        <v>131</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15">
+        <v>12</v>
+      </c>
+      <c r="P15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>300</v>
+      </c>
+      <c r="R15">
+        <v>27</v>
+      </c>
+      <c r="S15" t="s">
+        <v>301</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="U15" t="s">
+        <v>303</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W15" t="s">
+        <v>304</v>
+      </c>
+      <c r="X15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>305</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>307</v>
+      </c>
+      <c r="D16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E16" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>130</v>
+      </c>
+      <c r="I16">
+        <v>10.8</v>
+      </c>
+      <c r="J16">
+        <v>15.7</v>
+      </c>
+      <c r="K16" t="s">
+        <v>235</v>
+      </c>
+      <c r="L16" t="s">
+        <v>236</v>
+      </c>
+      <c r="M16" t="s">
+        <v>131</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16">
+        <v>25</v>
+      </c>
+      <c r="P16" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>308</v>
+      </c>
+      <c r="R16">
+        <v>28</v>
+      </c>
+      <c r="S16" t="s">
+        <v>309</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="U16" t="s">
+        <v>310</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" t="s">
+        <v>311</v>
+      </c>
+      <c r="X16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>312</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>314</v>
+      </c>
+      <c r="D17" t="s">
+        <v>184</v>
+      </c>
+      <c r="E17" t="s">
+        <v>185</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" t="s">
+        <v>186</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>9.8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>235</v>
+      </c>
+      <c r="L17" t="s">
+        <v>236</v>
+      </c>
+      <c r="M17" t="s">
+        <v>38</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17" t="s">
+        <v>187</v>
+      </c>
+      <c r="P17" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17">
+        <v>20</v>
+      </c>
+      <c r="S17" t="s">
+        <v>315</v>
+      </c>
+      <c r="T17" t="s">
+        <v>38</v>
+      </c>
+      <c r="U17" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" t="s">
+        <v>38</v>
+      </c>
+      <c r="W17" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>317</v>
+      </c>
+      <c r="D18" t="s">
+        <v>191</v>
+      </c>
+      <c r="E18" t="s">
+        <v>185</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>192</v>
+      </c>
+      <c r="H18" t="s">
+        <v>186</v>
+      </c>
+      <c r="I18">
+        <v>4.4</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>235</v>
+      </c>
+      <c r="L18" t="s">
+        <v>236</v>
+      </c>
+      <c r="M18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18" t="s">
+        <v>187</v>
+      </c>
+      <c r="P18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R18">
+        <v>8</v>
+      </c>
+      <c r="S18" t="s">
+        <v>318</v>
+      </c>
+      <c r="T18" t="s">
+        <v>38</v>
+      </c>
+      <c r="U18" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" t="s">
+        <v>38</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>320</v>
+      </c>
+      <c r="D19" t="s">
+        <v>196</v>
+      </c>
+      <c r="E19" t="s">
+        <v>185</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>109</v>
+      </c>
+      <c r="H19" t="s">
+        <v>197</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>235</v>
+      </c>
+      <c r="L19" t="s">
+        <v>236</v>
+      </c>
+      <c r="M19" t="s">
+        <v>38</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19" t="s">
+        <v>187</v>
+      </c>
+      <c r="P19" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19">
+        <v>17</v>
+      </c>
+      <c r="S19" t="s">
+        <v>321</v>
+      </c>
+      <c r="T19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U19" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" t="s">
+        <v>38</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>323</v>
+      </c>
+      <c r="D20" t="s">
+        <v>201</v>
+      </c>
+      <c r="E20" t="s">
+        <v>202</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>203</v>
+      </c>
+      <c r="H20" t="s">
+        <v>204</v>
+      </c>
+      <c r="I20">
+        <v>7.9</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>235</v>
+      </c>
+      <c r="L20" t="s">
+        <v>236</v>
+      </c>
+      <c r="M20" t="s">
+        <v>38</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20" t="s">
+        <v>187</v>
+      </c>
+      <c r="P20" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>38</v>
+      </c>
+      <c r="R20">
+        <v>21</v>
+      </c>
+      <c r="S20" t="s">
+        <v>324</v>
+      </c>
+      <c r="T20" t="s">
+        <v>38</v>
+      </c>
+      <c r="U20" t="s">
+        <v>38</v>
+      </c>
+      <c r="V20" t="s">
+        <v>38</v>
+      </c>
+      <c r="W20" t="s">
+        <v>38</v>
+      </c>
+      <c r="X20" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>326</v>
+      </c>
+      <c r="D21" t="s">
+        <v>213</v>
+      </c>
+      <c r="E21" t="s">
+        <v>202</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>214</v>
+      </c>
+      <c r="H21" t="s">
+        <v>204</v>
+      </c>
+      <c r="I21">
+        <v>3.7</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>235</v>
+      </c>
+      <c r="L21" t="s">
+        <v>236</v>
+      </c>
+      <c r="M21" t="s">
+        <v>38</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21" t="s">
+        <v>187</v>
+      </c>
+      <c r="P21" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>38</v>
+      </c>
+      <c r="R21">
+        <v>10</v>
+      </c>
+      <c r="S21" t="s">
+        <v>327</v>
+      </c>
+      <c r="T21" t="s">
+        <v>38</v>
+      </c>
+      <c r="U21" t="s">
+        <v>38</v>
+      </c>
+      <c r="V21" t="s">
+        <v>38</v>
+      </c>
+      <c r="W21" t="s">
+        <v>38</v>
+      </c>
+      <c r="X21" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>329</v>
+      </c>
+      <c r="D22" t="s">
+        <v>218</v>
+      </c>
+      <c r="E22" t="s">
+        <v>202</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>203</v>
+      </c>
+      <c r="H22" t="s">
+        <v>214</v>
+      </c>
+      <c r="I22">
+        <v>4.2</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>235</v>
+      </c>
+      <c r="L22" t="s">
+        <v>236</v>
+      </c>
+      <c r="M22" t="s">
+        <v>38</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22" t="s">
+        <v>187</v>
+      </c>
+      <c r="P22" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>38</v>
+      </c>
+      <c r="R22">
+        <v>11</v>
+      </c>
+      <c r="S22" t="s">
+        <v>330</v>
+      </c>
+      <c r="T22" t="s">
+        <v>38</v>
+      </c>
+      <c r="U22" t="s">
+        <v>38</v>
+      </c>
+      <c r="V22" t="s">
+        <v>38</v>
+      </c>
+      <c r="W22" t="s">
+        <v>38</v>
+      </c>
+      <c r="X22" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>332</v>
+      </c>
+      <c r="D23" t="s">
+        <v>222</v>
+      </c>
+      <c r="E23" t="s">
+        <v>202</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>203</v>
+      </c>
+      <c r="H23" t="s">
+        <v>223</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>235</v>
+      </c>
+      <c r="L23" t="s">
+        <v>236</v>
+      </c>
+      <c r="M23" t="s">
+        <v>38</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23" t="s">
+        <v>187</v>
+      </c>
+      <c r="P23" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>38</v>
+      </c>
+      <c r="R23">
+        <v>19</v>
+      </c>
+      <c r="S23" t="s">
+        <v>333</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" t="s">
+        <v>38</v>
+      </c>
+      <c r="W23" t="s">
+        <v>38</v>
+      </c>
+      <c r="X23" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>335</v>
+      </c>
+      <c r="D24" t="s">
+        <v>227</v>
+      </c>
+      <c r="E24" t="s">
+        <v>202</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>214</v>
+      </c>
+      <c r="H24" t="s">
+        <v>223</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>235</v>
+      </c>
+      <c r="L24" t="s">
+        <v>236</v>
+      </c>
+      <c r="M24" t="s">
+        <v>38</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24" t="s">
+        <v>187</v>
+      </c>
+      <c r="P24" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>38</v>
+      </c>
+      <c r="R24">
+        <v>8</v>
+      </c>
+      <c r="S24" t="s">
+        <v>336</v>
+      </c>
+      <c r="T24" t="s">
+        <v>38</v>
+      </c>
+      <c r="U24" t="s">
+        <v>38</v>
+      </c>
+      <c r="V24" t="s">
+        <v>38</v>
+      </c>
+      <c r="W24" t="s">
+        <v>38</v>
+      </c>
+      <c r="X24" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>338</v>
+      </c>
+      <c r="D25" t="s">
+        <v>231</v>
+      </c>
+      <c r="E25" t="s">
+        <v>202</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>223</v>
+      </c>
+      <c r="H25" t="s">
+        <v>204</v>
+      </c>
+      <c r="I25">
+        <v>1.3</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>235</v>
+      </c>
+      <c r="L25" t="s">
+        <v>236</v>
+      </c>
+      <c r="M25" t="s">
+        <v>38</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25" t="s">
+        <v>187</v>
+      </c>
+      <c r="P25" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>38</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s">
+        <v>339</v>
+      </c>
+      <c r="T25" t="s">
+        <v>38</v>
+      </c>
+      <c r="U25" t="s">
+        <v>38</v>
+      </c>
+      <c r="V25" t="s">
+        <v>38</v>
+      </c>
+      <c r="W25" t="s">
+        <v>38</v>
+      </c>
+      <c r="X25" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>340</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1"/>
+    <hyperlink ref="Y2" r:id="rId2"/>
+    <hyperlink ref="X3" r:id="rId3"/>
+    <hyperlink ref="Y3" r:id="rId4"/>
+    <hyperlink ref="Y4" r:id="rId5"/>
+    <hyperlink ref="Y5" r:id="rId6"/>
+    <hyperlink ref="Y6" r:id="rId7"/>
+    <hyperlink ref="X7" r:id="rId8"/>
+    <hyperlink ref="Y7" r:id="rId9"/>
+    <hyperlink ref="Y8" r:id="rId10"/>
+    <hyperlink ref="X9" r:id="rId11"/>
+    <hyperlink ref="Y9" r:id="rId12"/>
+    <hyperlink ref="X10" r:id="rId13"/>
+    <hyperlink ref="Y10" r:id="rId14"/>
+    <hyperlink ref="X11" r:id="rId15"/>
+    <hyperlink ref="Y11" r:id="rId16"/>
+    <hyperlink ref="Y12" r:id="rId17"/>
+    <hyperlink ref="Y13" r:id="rId18"/>
+    <hyperlink ref="Y14" r:id="rId19"/>
+    <hyperlink ref="X15" r:id="rId20"/>
+    <hyperlink ref="Y15" r:id="rId21"/>
+    <hyperlink ref="X16" r:id="rId22"/>
+    <hyperlink ref="Y16" r:id="rId23"/>
+    <hyperlink ref="Y17" r:id="rId24"/>
+    <hyperlink ref="Y18" r:id="rId25"/>
+    <hyperlink ref="Y19" r:id="rId26"/>
+    <hyperlink ref="Y20" r:id="rId27"/>
+    <hyperlink ref="Y21" r:id="rId28"/>
+    <hyperlink ref="Y22" r:id="rId29"/>
+    <hyperlink ref="Y23" r:id="rId30"/>
+    <hyperlink ref="Y24" r:id="rId31"/>
+    <hyperlink ref="Y25" r:id="rId32"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -3299,34 +5769,61 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>234</v>
+        <v>341</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>235</v>
+        <v>342</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>236</v>
+        <v>343</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>237</v>
+        <v>344</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>238</v>
+        <v>345</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>239</v>
+        <v>346</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>240</v>
+        <v>347</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>241</v>
+        <v>348</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>242</v>
+        <v>349</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>358</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -3372,8 +5869,35 @@
       <c r="O2" t="s">
         <v>44</v>
       </c>
+      <c r="P2" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2">
+        <v>30</v>
+      </c>
+      <c r="T2" t="s">
+        <v>39</v>
+      </c>
+      <c r="U2" t="s">
+        <v>237</v>
+      </c>
+      <c r="V2">
+        <v>35</v>
+      </c>
+      <c r="W2" t="s">
+        <v>39</v>
+      </c>
+      <c r="X2" t="s">
+        <v>241</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -3419,8 +5943,35 @@
       <c r="O3" t="s">
         <v>55</v>
       </c>
+      <c r="P3" t="s">
+        <v>244</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>38</v>
+      </c>
+      <c r="S3">
+        <v>33</v>
+      </c>
+      <c r="T3" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3" t="s">
+        <v>245</v>
+      </c>
+      <c r="V3">
+        <v>47</v>
+      </c>
+      <c r="W3" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3" t="s">
+        <v>248</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -3466,8 +6017,35 @@
       <c r="O4" t="s">
         <v>67</v>
       </c>
+      <c r="P4" t="s">
+        <v>251</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R4" t="s">
+        <v>38</v>
+      </c>
+      <c r="S4" t="s">
+        <v>187</v>
+      </c>
+      <c r="T4" t="s">
+        <v>38</v>
+      </c>
+      <c r="U4" t="s">
+        <v>38</v>
+      </c>
+      <c r="V4">
+        <v>16</v>
+      </c>
+      <c r="W4" t="s">
+        <v>38</v>
+      </c>
+      <c r="X4" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -3513,8 +6091,35 @@
       <c r="O5" t="s">
         <v>76</v>
       </c>
+      <c r="P5" t="s">
+        <v>253</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>38</v>
+      </c>
+      <c r="R5" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5" t="s">
+        <v>187</v>
+      </c>
+      <c r="T5" t="s">
+        <v>38</v>
+      </c>
+      <c r="U5" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5">
+        <v>18</v>
+      </c>
+      <c r="W5" t="s">
+        <v>38</v>
+      </c>
+      <c r="X5" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -3560,8 +6165,35 @@
       <c r="O6" t="s">
         <v>86</v>
       </c>
+      <c r="P6" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>38</v>
+      </c>
+      <c r="R6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S6" t="s">
+        <v>187</v>
+      </c>
+      <c r="T6" t="s">
+        <v>38</v>
+      </c>
+      <c r="U6" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6">
+        <v>16</v>
+      </c>
+      <c r="W6" t="s">
+        <v>38</v>
+      </c>
+      <c r="X6" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -3607,8 +6239,35 @@
       <c r="O7" t="s">
         <v>94</v>
       </c>
+      <c r="P7" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>37</v>
+      </c>
+      <c r="R7" t="s">
+        <v>38</v>
+      </c>
+      <c r="S7">
+        <v>14</v>
+      </c>
+      <c r="T7" t="s">
+        <v>39</v>
+      </c>
+      <c r="U7" t="s">
+        <v>260</v>
+      </c>
+      <c r="V7">
+        <v>18</v>
+      </c>
+      <c r="W7" t="s">
+        <v>39</v>
+      </c>
+      <c r="X7" t="s">
+        <v>264</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>98</v>
       </c>
@@ -3654,8 +6313,35 @@
       <c r="O8" t="s">
         <v>104</v>
       </c>
+      <c r="P8" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>38</v>
+      </c>
+      <c r="R8" t="s">
+        <v>38</v>
+      </c>
+      <c r="S8" t="s">
+        <v>187</v>
+      </c>
+      <c r="T8" t="s">
+        <v>38</v>
+      </c>
+      <c r="U8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V8">
+        <v>24</v>
+      </c>
+      <c r="W8" t="s">
+        <v>38</v>
+      </c>
+      <c r="X8" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>108</v>
       </c>
@@ -3701,8 +6387,35 @@
       <c r="O9" t="s">
         <v>114</v>
       </c>
+      <c r="P9" t="s">
+        <v>270</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>37</v>
+      </c>
+      <c r="R9" t="s">
+        <v>38</v>
+      </c>
+      <c r="S9">
+        <v>17</v>
+      </c>
+      <c r="T9" t="s">
+        <v>39</v>
+      </c>
+      <c r="U9" t="s">
+        <v>271</v>
+      </c>
+      <c r="V9">
+        <v>20</v>
+      </c>
+      <c r="W9" t="s">
+        <v>39</v>
+      </c>
+      <c r="X9" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -3748,8 +6461,35 @@
       <c r="O10" t="s">
         <v>123</v>
       </c>
+      <c r="P10" t="s">
+        <v>278</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>37</v>
+      </c>
+      <c r="R10" t="s">
+        <v>38</v>
+      </c>
+      <c r="S10">
+        <v>16</v>
+      </c>
+      <c r="T10" t="s">
+        <v>39</v>
+      </c>
+      <c r="U10" t="s">
+        <v>279</v>
+      </c>
+      <c r="V10">
+        <v>29</v>
+      </c>
+      <c r="W10" t="s">
+        <v>39</v>
+      </c>
+      <c r="X10" t="s">
+        <v>282</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>127</v>
       </c>
@@ -3795,8 +6535,35 @@
       <c r="O11" t="s">
         <v>135</v>
       </c>
+      <c r="P11" t="s">
+        <v>285</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>131</v>
+      </c>
+      <c r="R11" t="s">
+        <v>38</v>
+      </c>
+      <c r="S11">
+        <v>30</v>
+      </c>
+      <c r="T11" t="s">
+        <v>39</v>
+      </c>
+      <c r="U11" t="s">
+        <v>286</v>
+      </c>
+      <c r="V11">
+        <v>35</v>
+      </c>
+      <c r="W11" t="s">
+        <v>39</v>
+      </c>
+      <c r="X11" t="s">
+        <v>241</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>139</v>
       </c>
@@ -3842,8 +6609,35 @@
       <c r="O12" t="s">
         <v>144</v>
       </c>
+      <c r="P12" t="s">
+        <v>290</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>38</v>
+      </c>
+      <c r="R12" t="s">
+        <v>38</v>
+      </c>
+      <c r="S12" t="s">
+        <v>187</v>
+      </c>
+      <c r="T12" t="s">
+        <v>38</v>
+      </c>
+      <c r="U12" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12">
+        <v>21</v>
+      </c>
+      <c r="W12" t="s">
+        <v>38</v>
+      </c>
+      <c r="X12" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>148</v>
       </c>
@@ -3889,8 +6683,35 @@
       <c r="O13" t="s">
         <v>153</v>
       </c>
+      <c r="P13" t="s">
+        <v>293</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>38</v>
+      </c>
+      <c r="R13" t="s">
+        <v>38</v>
+      </c>
+      <c r="S13" t="s">
+        <v>187</v>
+      </c>
+      <c r="T13" t="s">
+        <v>38</v>
+      </c>
+      <c r="U13" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13">
+        <v>28</v>
+      </c>
+      <c r="W13" t="s">
+        <v>38</v>
+      </c>
+      <c r="X13" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>157</v>
       </c>
@@ -3936,8 +6757,35 @@
       <c r="O14" t="s">
         <v>164</v>
       </c>
+      <c r="P14" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>38</v>
+      </c>
+      <c r="R14" t="s">
+        <v>38</v>
+      </c>
+      <c r="S14" t="s">
+        <v>187</v>
+      </c>
+      <c r="T14" t="s">
+        <v>38</v>
+      </c>
+      <c r="U14" t="s">
+        <v>38</v>
+      </c>
+      <c r="V14">
+        <v>16</v>
+      </c>
+      <c r="W14" t="s">
+        <v>38</v>
+      </c>
+      <c r="X14" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>168</v>
       </c>
@@ -3983,8 +6831,35 @@
       <c r="O15" t="s">
         <v>172</v>
       </c>
+      <c r="P15" t="s">
+        <v>299</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>131</v>
+      </c>
+      <c r="R15" t="s">
+        <v>38</v>
+      </c>
+      <c r="S15">
+        <v>12</v>
+      </c>
+      <c r="T15" t="s">
+        <v>39</v>
+      </c>
+      <c r="U15" t="s">
+        <v>300</v>
+      </c>
+      <c r="V15">
+        <v>27</v>
+      </c>
+      <c r="W15" t="s">
+        <v>39</v>
+      </c>
+      <c r="X15" t="s">
+        <v>304</v>
+      </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>176</v>
       </c>
@@ -4030,8 +6905,35 @@
       <c r="O16" t="s">
         <v>180</v>
       </c>
+      <c r="P16" t="s">
+        <v>307</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>131</v>
+      </c>
+      <c r="R16" t="s">
+        <v>38</v>
+      </c>
+      <c r="S16">
+        <v>25</v>
+      </c>
+      <c r="T16" t="s">
+        <v>39</v>
+      </c>
+      <c r="U16" t="s">
+        <v>308</v>
+      </c>
+      <c r="V16">
+        <v>28</v>
+      </c>
+      <c r="W16" t="s">
+        <v>39</v>
+      </c>
+      <c r="X16" t="s">
+        <v>311</v>
+      </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>184</v>
       </c>
@@ -4077,8 +6979,35 @@
       <c r="O17" t="s">
         <v>38</v>
       </c>
+      <c r="P17" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17" t="s">
+        <v>38</v>
+      </c>
+      <c r="S17" t="s">
+        <v>187</v>
+      </c>
+      <c r="T17" t="s">
+        <v>38</v>
+      </c>
+      <c r="U17" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17">
+        <v>20</v>
+      </c>
+      <c r="W17" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>191</v>
       </c>
@@ -4124,8 +7053,35 @@
       <c r="O18" t="s">
         <v>38</v>
       </c>
+      <c r="P18" t="s">
+        <v>317</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R18" t="s">
+        <v>38</v>
+      </c>
+      <c r="S18" t="s">
+        <v>187</v>
+      </c>
+      <c r="T18" t="s">
+        <v>38</v>
+      </c>
+      <c r="U18" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18">
+        <v>8</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>196</v>
       </c>
@@ -4171,8 +7127,35 @@
       <c r="O19" t="s">
         <v>38</v>
       </c>
+      <c r="P19" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19" t="s">
+        <v>38</v>
+      </c>
+      <c r="S19" t="s">
+        <v>187</v>
+      </c>
+      <c r="T19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U19" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19">
+        <v>17</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>201</v>
       </c>
@@ -4218,8 +7201,35 @@
       <c r="O20" t="s">
         <v>209</v>
       </c>
+      <c r="P20" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>38</v>
+      </c>
+      <c r="R20" t="s">
+        <v>38</v>
+      </c>
+      <c r="S20" t="s">
+        <v>187</v>
+      </c>
+      <c r="T20" t="s">
+        <v>38</v>
+      </c>
+      <c r="U20" t="s">
+        <v>38</v>
+      </c>
+      <c r="V20">
+        <v>21</v>
+      </c>
+      <c r="W20" t="s">
+        <v>38</v>
+      </c>
+      <c r="X20" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>213</v>
       </c>
@@ -4265,8 +7275,35 @@
       <c r="O21" t="s">
         <v>38</v>
       </c>
+      <c r="P21" t="s">
+        <v>326</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>38</v>
+      </c>
+      <c r="R21" t="s">
+        <v>38</v>
+      </c>
+      <c r="S21" t="s">
+        <v>187</v>
+      </c>
+      <c r="T21" t="s">
+        <v>38</v>
+      </c>
+      <c r="U21" t="s">
+        <v>38</v>
+      </c>
+      <c r="V21">
+        <v>10</v>
+      </c>
+      <c r="W21" t="s">
+        <v>38</v>
+      </c>
+      <c r="X21" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>218</v>
       </c>
@@ -4312,8 +7349,35 @@
       <c r="O22" t="s">
         <v>38</v>
       </c>
+      <c r="P22" t="s">
+        <v>329</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>38</v>
+      </c>
+      <c r="R22" t="s">
+        <v>38</v>
+      </c>
+      <c r="S22" t="s">
+        <v>187</v>
+      </c>
+      <c r="T22" t="s">
+        <v>38</v>
+      </c>
+      <c r="U22" t="s">
+        <v>38</v>
+      </c>
+      <c r="V22">
+        <v>11</v>
+      </c>
+      <c r="W22" t="s">
+        <v>38</v>
+      </c>
+      <c r="X22" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>222</v>
       </c>
@@ -4359,8 +7423,35 @@
       <c r="O23" t="s">
         <v>38</v>
       </c>
+      <c r="P23" t="s">
+        <v>332</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>38</v>
+      </c>
+      <c r="R23" t="s">
+        <v>38</v>
+      </c>
+      <c r="S23" t="s">
+        <v>187</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23">
+        <v>19</v>
+      </c>
+      <c r="W23" t="s">
+        <v>38</v>
+      </c>
+      <c r="X23" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>227</v>
       </c>
@@ -4406,8 +7497,35 @@
       <c r="O24" t="s">
         <v>38</v>
       </c>
+      <c r="P24" t="s">
+        <v>335</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>38</v>
+      </c>
+      <c r="R24" t="s">
+        <v>38</v>
+      </c>
+      <c r="S24" t="s">
+        <v>187</v>
+      </c>
+      <c r="T24" t="s">
+        <v>38</v>
+      </c>
+      <c r="U24" t="s">
+        <v>38</v>
+      </c>
+      <c r="V24">
+        <v>8</v>
+      </c>
+      <c r="W24" t="s">
+        <v>38</v>
+      </c>
+      <c r="X24" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>231</v>
       </c>
@@ -4453,9 +7571,36 @@
       <c r="O25" t="s">
         <v>38</v>
       </c>
+      <c r="P25" t="s">
+        <v>338</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>38</v>
+      </c>
+      <c r="R25" t="s">
+        <v>38</v>
+      </c>
+      <c r="S25" t="s">
+        <v>187</v>
+      </c>
+      <c r="T25" t="s">
+        <v>38</v>
+      </c>
+      <c r="U25" t="s">
+        <v>38</v>
+      </c>
+      <c r="V25">
+        <v>3</v>
+      </c>
+      <c r="W25" t="s">
+        <v>38</v>
+      </c>
+      <c r="X25" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:X1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Auto-collect traffic data: 2026-10-19 01:16 PM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-10-19_Mon.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-10-19_Mon.xlsx
@@ -6,14 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="1_00 PM" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="All Periods Combined" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2426" uniqueCount="528">
   <si>
     <t>Date</t>
   </si>
@@ -1038,6 +1039,486 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/10_00_AM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>10/19/2026, 1:03:23 PM</t>
+  </si>
+  <si>
+    <t>1:00 PM</t>
+  </si>
+  <si>
+    <t>Monday (Weekday) - Mid-day Off-Peak</t>
+  </si>
+  <si>
+    <t> | 28 min | 1:08 AM—1:36 AM | Blue Line | 1:08 AM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 47 min | 12.4 km | via Barrackpore Trunk Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>19 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.68x</t>
+  </si>
+  <si>
+    <t>40.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:03:42 PM</t>
+  </si>
+  <si>
+    <t> | 28 min | 1:07 AM—1:35 AM | Blue Line | 1:07 AM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 59 min | 14.7 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>31 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.11x</t>
+  </si>
+  <si>
+    <t>52.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:04:00 PM</t>
+  </si>
+  <si>
+    <t> | 7 min | 1:00 AM—1:07 AM | Blue Line | 1:00 AM from Shyambazar | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 18 min | 4.1 km | via Belgachia Rd/Khudiram Bose Sarani | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>11 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.57x</t>
+  </si>
+  <si>
+    <t>61.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:04:20 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 1:05 AM—1:16 AM | Blue Line | 1:05 AM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 27 min | 5.2 km | via Jatindra Mohan Ave and Central Ave/Chittaranjan Ave | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>16 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.45x</t>
+  </si>
+  <si>
+    <t>59.3% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:04:39 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 1:00 AM—1:11 AM | Blue Line | 1:00 AM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 18 min | 5.1 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:04:58 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 1:08 AM—1:20 AM | Blue Line | 1:08 AM from Dakshineswar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 22 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.83x</t>
+  </si>
+  <si>
+    <t>45.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:05:17 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 1:00 AM—1:18 AM | Blue Line | 1:00 AM from Esplanade | ₹15.00  1 min | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 8.3 km | via Chowringee Rd/Jawaharlal Nehru Rd and Ashutosh Mukherjee Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.56x</t>
+  </si>
+  <si>
+    <t>35.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:05:36 PM</t>
+  </si>
+  <si>
+    <t> | 16 min | 1:03 AM—1:19 AM | Blue Line | 1:04 AM from Mahanayak Uttamkumar | ₹15.00  1 min | Details</t>
+  </si>
+  <si>
+    <t> | 26 min | 6.4 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.63x</t>
+  </si>
+  <si>
+    <t>38.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:05:55 PM</t>
+  </si>
+  <si>
+    <t> | 16 min | 1:00 AM—1:16 AM | Blue Line | 1:00 AM from Dumdum | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 38 min | 8.8 km | via Jessore Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>22 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.38x</t>
+  </si>
+  <si>
+    <t>57.9% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:06:14 PM</t>
+  </si>
+  <si>
+    <t> | 30 min | 1:04 AM—1:34 AM | Green Line | 1:04 AM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 40 min | 10.8 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.33x</t>
+  </si>
+  <si>
+    <t>25.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:06:33 PM</t>
+  </si>
+  <si>
+    <t> | 21 min | 1:03 AM—1:24 AM | Green Line | 1:03 AM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 23 min | 8.0 km | via Beleghata Main Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>2 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.10x</t>
+  </si>
+  <si>
+    <t>8.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:06:50 PM</t>
+  </si>
+  <si>
+    <t> | 9 min | 1:04 AM—1:13 AM | Green Line | 1:04 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 33 min | 7.2 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>24 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>3.67x</t>
+  </si>
+  <si>
+    <t>72.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:07:10 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 1:06 AM—1:24 AM | Green Line | 1:06 AM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 17 min | 5.4 km | via Narkeldanga Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.94x</t>
+  </si>
+  <si>
+    <t>5.6% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:07:30 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 1:04 AM—1:16 AM | Green Line | 1:04 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 32 min | 7.6 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>2.67x</t>
+  </si>
+  <si>
+    <t>62.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:07:50 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 1:09 AM—1:34 AM | Green Line | 1:09 AM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 12.4 km | via Jawaharlal Nehru Rd and Park St | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:09:33 PM</t>
+  </si>
+  <si>
+    <t> | 21 min | 9.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:11:16 PM</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:13:01 PM</t>
+  </si>
+  <si>
+    <t> | 19 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:13:34 PM</t>
+  </si>
+  <si>
+    <t> | 19 min | 3:00 PM—3:19 PM | Purple Line | 3:00 PM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 23 min | 7.8 km | via NH 12 | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.21x</t>
+  </si>
+  <si>
+    <t>17.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-19/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:13:53 PM</t>
+  </si>
+  <si>
+    <t> | 54 min | 3.9 km | via NH 12</t>
+  </si>
+  <si>
+    <t> | 12 min | 3.7 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>42 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.22x</t>
+  </si>
+  <si>
+    <t>77.8% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-20/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:14:12 PM</t>
+  </si>
+  <si>
+    <t> | 57 min | 4.1 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t> | 12 min | 4.1 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>45 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.21x</t>
+  </si>
+  <si>
+    <t>78.9% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-21/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:15:54 PM</t>
+  </si>
+  <si>
+    <t> | 21 min | 6.5 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:16:13 PM</t>
+  </si>
+  <si>
+    <t> | 33 min | 2.4 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t> | 9 min | 2.4 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>24 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.27x</t>
+  </si>
+  <si>
+    <t>72.7% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-23/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 1:16:32 PM</t>
+  </si>
+  <si>
+    <t> | 22 min | 1.5 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t>19 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.14x</t>
+  </si>
+  <si>
+    <t>86.4% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-24/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -1090,6 +1571,33 @@
   </si>
   <si>
     <t>10:00 AM Savings (%)</t>
+  </si>
+  <si>
+    <t>1:00 PM Scraped At</t>
+  </si>
+  <si>
+    <t>1:00 PM Actual Metro</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Walk</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro (min)</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Route</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>1:00 PM Car (min)</t>
+  </si>
+  <si>
+    <t>1:00 PM Faster Mode</t>
+  </si>
+  <si>
+    <t>1:00 PM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -5746,10 +6254,2143 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>12.4</v>
+      </c>
+      <c r="K2" t="s">
+        <v>342</v>
+      </c>
+      <c r="L2" t="s">
+        <v>343</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>344</v>
+      </c>
+      <c r="R2">
+        <v>47</v>
+      </c>
+      <c r="S2" t="s">
+        <v>345</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="U2" t="s">
+        <v>347</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" t="s">
+        <v>348</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>349</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>351</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.8</v>
+      </c>
+      <c r="J3">
+        <v>14.7</v>
+      </c>
+      <c r="K3" t="s">
+        <v>342</v>
+      </c>
+      <c r="L3" t="s">
+        <v>343</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3">
+        <v>28</v>
+      </c>
+      <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>352</v>
+      </c>
+      <c r="R3">
+        <v>59</v>
+      </c>
+      <c r="S3" t="s">
+        <v>353</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="U3" t="s">
+        <v>355</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>356</v>
+      </c>
+      <c r="X3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>357</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>359</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>4.3</v>
+      </c>
+      <c r="J4">
+        <v>4.1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>342</v>
+      </c>
+      <c r="L4" t="s">
+        <v>343</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4">
+        <v>7</v>
+      </c>
+      <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>360</v>
+      </c>
+      <c r="R4">
+        <v>18</v>
+      </c>
+      <c r="S4" t="s">
+        <v>361</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="U4" t="s">
+        <v>363</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W4" t="s">
+        <v>364</v>
+      </c>
+      <c r="X4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>367</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>5.2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>342</v>
+      </c>
+      <c r="L5" t="s">
+        <v>343</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5">
+        <v>11</v>
+      </c>
+      <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>368</v>
+      </c>
+      <c r="R5">
+        <v>27</v>
+      </c>
+      <c r="S5" t="s">
+        <v>369</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="U5" t="s">
+        <v>371</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W5" t="s">
+        <v>372</v>
+      </c>
+      <c r="X5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>373</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>375</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>342</v>
+      </c>
+      <c r="L6" t="s">
+        <v>343</v>
+      </c>
+      <c r="M6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6">
+        <v>11</v>
+      </c>
+      <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>376</v>
+      </c>
+      <c r="R6">
+        <v>18</v>
+      </c>
+      <c r="S6" t="s">
+        <v>377</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="U6" t="s">
+        <v>85</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W6" t="s">
+        <v>86</v>
+      </c>
+      <c r="X6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>378</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>380</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>6.2</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>342</v>
+      </c>
+      <c r="L7" t="s">
+        <v>343</v>
+      </c>
+      <c r="M7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>12</v>
+      </c>
+      <c r="P7" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>381</v>
+      </c>
+      <c r="R7">
+        <v>22</v>
+      </c>
+      <c r="S7" t="s">
+        <v>382</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="U7" t="s">
+        <v>383</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>384</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>385</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>387</v>
+      </c>
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>99</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>8.3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>342</v>
+      </c>
+      <c r="L8" t="s">
+        <v>343</v>
+      </c>
+      <c r="M8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8">
+        <v>18</v>
+      </c>
+      <c r="P8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>388</v>
+      </c>
+      <c r="R8">
+        <v>28</v>
+      </c>
+      <c r="S8" t="s">
+        <v>389</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="U8" t="s">
+        <v>390</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W8" t="s">
+        <v>391</v>
+      </c>
+      <c r="X8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>392</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>394</v>
+      </c>
+      <c r="D9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>99</v>
+      </c>
+      <c r="H9" t="s">
+        <v>109</v>
+      </c>
+      <c r="I9">
+        <v>7.1</v>
+      </c>
+      <c r="J9">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="s">
+        <v>342</v>
+      </c>
+      <c r="L9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9">
+        <v>16</v>
+      </c>
+      <c r="P9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>395</v>
+      </c>
+      <c r="R9">
+        <v>26</v>
+      </c>
+      <c r="S9" t="s">
+        <v>396</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="U9" t="s">
+        <v>397</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W9" t="s">
+        <v>398</v>
+      </c>
+      <c r="X9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>399</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>401</v>
+      </c>
+      <c r="D10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>8.8</v>
+      </c>
+      <c r="J10">
+        <v>8.8</v>
+      </c>
+      <c r="K10" t="s">
+        <v>342</v>
+      </c>
+      <c r="L10" t="s">
+        <v>343</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10">
+        <v>16</v>
+      </c>
+      <c r="P10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>402</v>
+      </c>
+      <c r="R10">
+        <v>38</v>
+      </c>
+      <c r="S10" t="s">
+        <v>403</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="U10" t="s">
+        <v>405</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W10" t="s">
+        <v>406</v>
+      </c>
+      <c r="X10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>407</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>409</v>
+      </c>
+      <c r="D11" t="s">
+        <v>127</v>
+      </c>
+      <c r="E11" t="s">
+        <v>128</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" t="s">
+        <v>130</v>
+      </c>
+      <c r="I11">
+        <v>14.2</v>
+      </c>
+      <c r="J11">
+        <v>10.8</v>
+      </c>
+      <c r="K11" t="s">
+        <v>342</v>
+      </c>
+      <c r="L11" t="s">
+        <v>343</v>
+      </c>
+      <c r="M11" t="s">
+        <v>131</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11">
+        <v>30</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>410</v>
+      </c>
+      <c r="R11">
+        <v>40</v>
+      </c>
+      <c r="S11" t="s">
+        <v>411</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="U11" t="s">
+        <v>412</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W11" t="s">
+        <v>413</v>
+      </c>
+      <c r="X11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>414</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>416</v>
+      </c>
+      <c r="D12" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" t="s">
+        <v>128</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>140</v>
+      </c>
+      <c r="H12" t="s">
+        <v>130</v>
+      </c>
+      <c r="I12">
+        <v>8.3</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>342</v>
+      </c>
+      <c r="L12" t="s">
+        <v>343</v>
+      </c>
+      <c r="M12" t="s">
+        <v>131</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12">
+        <v>21</v>
+      </c>
+      <c r="P12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>417</v>
+      </c>
+      <c r="R12">
+        <v>23</v>
+      </c>
+      <c r="S12" t="s">
+        <v>418</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="U12" t="s">
+        <v>420</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W12" t="s">
+        <v>421</v>
+      </c>
+      <c r="X12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>422</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>424</v>
+      </c>
+      <c r="D13" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" t="s">
+        <v>128</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" t="s">
+        <v>140</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>7.2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>342</v>
+      </c>
+      <c r="L13" t="s">
+        <v>343</v>
+      </c>
+      <c r="M13" t="s">
+        <v>131</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13">
+        <v>9</v>
+      </c>
+      <c r="P13" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>425</v>
+      </c>
+      <c r="R13">
+        <v>33</v>
+      </c>
+      <c r="S13" t="s">
+        <v>426</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="U13" t="s">
+        <v>428</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W13" t="s">
+        <v>429</v>
+      </c>
+      <c r="X13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>430</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>432</v>
+      </c>
+      <c r="D14" t="s">
+        <v>157</v>
+      </c>
+      <c r="E14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>158</v>
+      </c>
+      <c r="H14" t="s">
+        <v>130</v>
+      </c>
+      <c r="I14">
+        <v>7.3</v>
+      </c>
+      <c r="J14">
+        <v>5.4</v>
+      </c>
+      <c r="K14" t="s">
+        <v>342</v>
+      </c>
+      <c r="L14" t="s">
+        <v>343</v>
+      </c>
+      <c r="M14" t="s">
+        <v>131</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14">
+        <v>18</v>
+      </c>
+      <c r="P14" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>433</v>
+      </c>
+      <c r="R14">
+        <v>17</v>
+      </c>
+      <c r="S14" t="s">
+        <v>434</v>
+      </c>
+      <c r="T14" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="U14" t="s">
+        <v>436</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="W14" t="s">
+        <v>437</v>
+      </c>
+      <c r="X14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>438</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>440</v>
+      </c>
+      <c r="D15" t="s">
+        <v>168</v>
+      </c>
+      <c r="E15" t="s">
+        <v>128</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" t="s">
+        <v>158</v>
+      </c>
+      <c r="I15">
+        <v>7.7</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>342</v>
+      </c>
+      <c r="L15" t="s">
+        <v>343</v>
+      </c>
+      <c r="M15" t="s">
+        <v>131</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15">
+        <v>12</v>
+      </c>
+      <c r="P15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>441</v>
+      </c>
+      <c r="R15">
+        <v>32</v>
+      </c>
+      <c r="S15" t="s">
+        <v>442</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="U15" t="s">
+        <v>443</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W15" t="s">
+        <v>444</v>
+      </c>
+      <c r="X15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>445</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>447</v>
+      </c>
+      <c r="D16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E16" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>130</v>
+      </c>
+      <c r="I16">
+        <v>11.3</v>
+      </c>
+      <c r="J16">
+        <v>12.4</v>
+      </c>
+      <c r="K16" t="s">
+        <v>342</v>
+      </c>
+      <c r="L16" t="s">
+        <v>343</v>
+      </c>
+      <c r="M16" t="s">
+        <v>131</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16">
+        <v>25</v>
+      </c>
+      <c r="P16" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>448</v>
+      </c>
+      <c r="R16">
+        <v>28</v>
+      </c>
+      <c r="S16" t="s">
+        <v>449</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="U16" t="s">
+        <v>310</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" t="s">
+        <v>311</v>
+      </c>
+      <c r="X16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>450</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>452</v>
+      </c>
+      <c r="D17" t="s">
+        <v>184</v>
+      </c>
+      <c r="E17" t="s">
+        <v>185</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" t="s">
+        <v>186</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>9.8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>342</v>
+      </c>
+      <c r="L17" t="s">
+        <v>343</v>
+      </c>
+      <c r="M17" t="s">
+        <v>38</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17" t="s">
+        <v>187</v>
+      </c>
+      <c r="P17" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17">
+        <v>21</v>
+      </c>
+      <c r="S17" t="s">
+        <v>453</v>
+      </c>
+      <c r="T17" t="s">
+        <v>38</v>
+      </c>
+      <c r="U17" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" t="s">
+        <v>38</v>
+      </c>
+      <c r="W17" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>455</v>
+      </c>
+      <c r="D18" t="s">
+        <v>191</v>
+      </c>
+      <c r="E18" t="s">
+        <v>185</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>192</v>
+      </c>
+      <c r="H18" t="s">
+        <v>186</v>
+      </c>
+      <c r="I18">
+        <v>4.4</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>342</v>
+      </c>
+      <c r="L18" t="s">
+        <v>343</v>
+      </c>
+      <c r="M18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18" t="s">
+        <v>187</v>
+      </c>
+      <c r="P18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R18">
+        <v>8</v>
+      </c>
+      <c r="S18" t="s">
+        <v>318</v>
+      </c>
+      <c r="T18" t="s">
+        <v>38</v>
+      </c>
+      <c r="U18" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" t="s">
+        <v>38</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>457</v>
+      </c>
+      <c r="D19" t="s">
+        <v>196</v>
+      </c>
+      <c r="E19" t="s">
+        <v>185</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>109</v>
+      </c>
+      <c r="H19" t="s">
+        <v>197</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>342</v>
+      </c>
+      <c r="L19" t="s">
+        <v>343</v>
+      </c>
+      <c r="M19" t="s">
+        <v>38</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19" t="s">
+        <v>187</v>
+      </c>
+      <c r="P19" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19">
+        <v>19</v>
+      </c>
+      <c r="S19" t="s">
+        <v>458</v>
+      </c>
+      <c r="T19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U19" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" t="s">
+        <v>38</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>460</v>
+      </c>
+      <c r="D20" t="s">
+        <v>201</v>
+      </c>
+      <c r="E20" t="s">
+        <v>202</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>203</v>
+      </c>
+      <c r="H20" t="s">
+        <v>204</v>
+      </c>
+      <c r="I20">
+        <v>8.6</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>342</v>
+      </c>
+      <c r="L20" t="s">
+        <v>343</v>
+      </c>
+      <c r="M20" t="s">
+        <v>205</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20">
+        <v>19</v>
+      </c>
+      <c r="P20" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>461</v>
+      </c>
+      <c r="R20">
+        <v>23</v>
+      </c>
+      <c r="S20" t="s">
+        <v>462</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="U20" t="s">
+        <v>463</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W20" t="s">
+        <v>464</v>
+      </c>
+      <c r="X20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>465</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>467</v>
+      </c>
+      <c r="D21" t="s">
+        <v>213</v>
+      </c>
+      <c r="E21" t="s">
+        <v>202</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>214</v>
+      </c>
+      <c r="H21" t="s">
+        <v>204</v>
+      </c>
+      <c r="I21">
+        <v>3.9</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>342</v>
+      </c>
+      <c r="L21" t="s">
+        <v>343</v>
+      </c>
+      <c r="M21" t="s">
+        <v>38</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21">
+        <v>54</v>
+      </c>
+      <c r="P21" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>468</v>
+      </c>
+      <c r="R21">
+        <v>12</v>
+      </c>
+      <c r="S21" t="s">
+        <v>469</v>
+      </c>
+      <c r="T21" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="U21" t="s">
+        <v>471</v>
+      </c>
+      <c r="V21" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="W21" t="s">
+        <v>472</v>
+      </c>
+      <c r="X21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>473</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>475</v>
+      </c>
+      <c r="D22" t="s">
+        <v>218</v>
+      </c>
+      <c r="E22" t="s">
+        <v>202</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>203</v>
+      </c>
+      <c r="H22" t="s">
+        <v>214</v>
+      </c>
+      <c r="I22">
+        <v>4.1</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>342</v>
+      </c>
+      <c r="L22" t="s">
+        <v>343</v>
+      </c>
+      <c r="M22" t="s">
+        <v>38</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22">
+        <v>57</v>
+      </c>
+      <c r="P22" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>476</v>
+      </c>
+      <c r="R22">
+        <v>12</v>
+      </c>
+      <c r="S22" t="s">
+        <v>477</v>
+      </c>
+      <c r="T22" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="U22" t="s">
+        <v>479</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="W22" t="s">
+        <v>480</v>
+      </c>
+      <c r="X22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>481</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>483</v>
+      </c>
+      <c r="D23" t="s">
+        <v>222</v>
+      </c>
+      <c r="E23" t="s">
+        <v>202</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>203</v>
+      </c>
+      <c r="H23" t="s">
+        <v>223</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>342</v>
+      </c>
+      <c r="L23" t="s">
+        <v>343</v>
+      </c>
+      <c r="M23" t="s">
+        <v>38</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23" t="s">
+        <v>187</v>
+      </c>
+      <c r="P23" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>38</v>
+      </c>
+      <c r="R23">
+        <v>21</v>
+      </c>
+      <c r="S23" t="s">
+        <v>484</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" t="s">
+        <v>38</v>
+      </c>
+      <c r="W23" t="s">
+        <v>38</v>
+      </c>
+      <c r="X23" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>486</v>
+      </c>
+      <c r="D24" t="s">
+        <v>227</v>
+      </c>
+      <c r="E24" t="s">
+        <v>202</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>214</v>
+      </c>
+      <c r="H24" t="s">
+        <v>223</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>342</v>
+      </c>
+      <c r="L24" t="s">
+        <v>343</v>
+      </c>
+      <c r="M24" t="s">
+        <v>38</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24">
+        <v>33</v>
+      </c>
+      <c r="P24" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>487</v>
+      </c>
+      <c r="R24">
+        <v>9</v>
+      </c>
+      <c r="S24" t="s">
+        <v>488</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="U24" t="s">
+        <v>490</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="W24" t="s">
+        <v>491</v>
+      </c>
+      <c r="X24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>492</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>494</v>
+      </c>
+      <c r="D25" t="s">
+        <v>231</v>
+      </c>
+      <c r="E25" t="s">
+        <v>202</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>223</v>
+      </c>
+      <c r="H25" t="s">
+        <v>204</v>
+      </c>
+      <c r="I25">
+        <v>1.5</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>342</v>
+      </c>
+      <c r="L25" t="s">
+        <v>343</v>
+      </c>
+      <c r="M25" t="s">
+        <v>38</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25">
+        <v>22</v>
+      </c>
+      <c r="P25" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>495</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s">
+        <v>232</v>
+      </c>
+      <c r="T25" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="U25" t="s">
+        <v>497</v>
+      </c>
+      <c r="V25" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="W25" t="s">
+        <v>498</v>
+      </c>
+      <c r="X25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>499</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>500</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1"/>
+    <hyperlink ref="Y2" r:id="rId2"/>
+    <hyperlink ref="X3" r:id="rId3"/>
+    <hyperlink ref="Y3" r:id="rId4"/>
+    <hyperlink ref="X4" r:id="rId5"/>
+    <hyperlink ref="Y4" r:id="rId6"/>
+    <hyperlink ref="X5" r:id="rId7"/>
+    <hyperlink ref="Y5" r:id="rId8"/>
+    <hyperlink ref="X6" r:id="rId9"/>
+    <hyperlink ref="Y6" r:id="rId10"/>
+    <hyperlink ref="X7" r:id="rId11"/>
+    <hyperlink ref="Y7" r:id="rId12"/>
+    <hyperlink ref="X8" r:id="rId13"/>
+    <hyperlink ref="Y8" r:id="rId14"/>
+    <hyperlink ref="X9" r:id="rId15"/>
+    <hyperlink ref="Y9" r:id="rId16"/>
+    <hyperlink ref="X10" r:id="rId17"/>
+    <hyperlink ref="Y10" r:id="rId18"/>
+    <hyperlink ref="X11" r:id="rId19"/>
+    <hyperlink ref="Y11" r:id="rId20"/>
+    <hyperlink ref="X12" r:id="rId21"/>
+    <hyperlink ref="Y12" r:id="rId22"/>
+    <hyperlink ref="X13" r:id="rId23"/>
+    <hyperlink ref="Y13" r:id="rId24"/>
+    <hyperlink ref="X14" r:id="rId25"/>
+    <hyperlink ref="Y14" r:id="rId26"/>
+    <hyperlink ref="X15" r:id="rId27"/>
+    <hyperlink ref="Y15" r:id="rId28"/>
+    <hyperlink ref="X16" r:id="rId29"/>
+    <hyperlink ref="Y16" r:id="rId30"/>
+    <hyperlink ref="Y17" r:id="rId31"/>
+    <hyperlink ref="Y18" r:id="rId32"/>
+    <hyperlink ref="Y19" r:id="rId33"/>
+    <hyperlink ref="X20" r:id="rId34"/>
+    <hyperlink ref="Y20" r:id="rId35"/>
+    <hyperlink ref="X21" r:id="rId36"/>
+    <hyperlink ref="Y21" r:id="rId37"/>
+    <hyperlink ref="X22" r:id="rId38"/>
+    <hyperlink ref="Y22" r:id="rId39"/>
+    <hyperlink ref="Y23" r:id="rId40"/>
+    <hyperlink ref="X24" r:id="rId41"/>
+    <hyperlink ref="Y24" r:id="rId42"/>
+    <hyperlink ref="X25" r:id="rId43"/>
+    <hyperlink ref="Y25" r:id="rId44"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AG25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:33" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -5769,61 +8410,88 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>341</v>
+        <v>501</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>342</v>
+        <v>502</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>343</v>
+        <v>503</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>344</v>
+        <v>504</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>345</v>
+        <v>505</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>346</v>
+        <v>506</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>347</v>
+        <v>507</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>348</v>
+        <v>508</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>349</v>
+        <v>509</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>350</v>
+        <v>510</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>351</v>
+        <v>511</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>352</v>
+        <v>512</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>353</v>
+        <v>513</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>354</v>
+        <v>514</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>355</v>
+        <v>515</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>356</v>
+        <v>516</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>357</v>
+        <v>517</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>358</v>
+        <v>518</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="AD1" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="AE1" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="AF1" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="AG1" s="4" t="s">
+        <v>527</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -5896,8 +8564,35 @@
       <c r="X2" t="s">
         <v>241</v>
       </c>
+      <c r="Y2" t="s">
+        <v>341</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB2">
+        <v>28</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>344</v>
+      </c>
+      <c r="AE2">
+        <v>47</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>348</v>
+      </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -5970,8 +8665,35 @@
       <c r="X3" t="s">
         <v>248</v>
       </c>
+      <c r="Y3" t="s">
+        <v>351</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB3">
+        <v>28</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>352</v>
+      </c>
+      <c r="AE3">
+        <v>59</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>356</v>
+      </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -6044,8 +8766,35 @@
       <c r="X4" t="s">
         <v>38</v>
       </c>
+      <c r="Y4" t="s">
+        <v>359</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB4">
+        <v>7</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>360</v>
+      </c>
+      <c r="AE4">
+        <v>18</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>364</v>
+      </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -6118,8 +8867,35 @@
       <c r="X5" t="s">
         <v>38</v>
       </c>
+      <c r="Y5" t="s">
+        <v>367</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB5">
+        <v>11</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>368</v>
+      </c>
+      <c r="AE5">
+        <v>27</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>372</v>
+      </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -6192,8 +8968,35 @@
       <c r="X6" t="s">
         <v>38</v>
       </c>
+      <c r="Y6" t="s">
+        <v>375</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB6">
+        <v>11</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>376</v>
+      </c>
+      <c r="AE6">
+        <v>18</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>86</v>
+      </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -6266,8 +9069,35 @@
       <c r="X7" t="s">
         <v>264</v>
       </c>
+      <c r="Y7" t="s">
+        <v>380</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB7">
+        <v>12</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>381</v>
+      </c>
+      <c r="AE7">
+        <v>22</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>384</v>
+      </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>98</v>
       </c>
@@ -6340,8 +9170,35 @@
       <c r="X8" t="s">
         <v>38</v>
       </c>
+      <c r="Y8" t="s">
+        <v>387</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB8">
+        <v>18</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>388</v>
+      </c>
+      <c r="AE8">
+        <v>28</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>391</v>
+      </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>108</v>
       </c>
@@ -6414,8 +9271,35 @@
       <c r="X9" t="s">
         <v>275</v>
       </c>
+      <c r="Y9" t="s">
+        <v>394</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB9">
+        <v>16</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>395</v>
+      </c>
+      <c r="AE9">
+        <v>26</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>398</v>
+      </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -6488,8 +9372,35 @@
       <c r="X10" t="s">
         <v>282</v>
       </c>
+      <c r="Y10" t="s">
+        <v>401</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB10">
+        <v>16</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>402</v>
+      </c>
+      <c r="AE10">
+        <v>38</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>406</v>
+      </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>127</v>
       </c>
@@ -6562,8 +9473,35 @@
       <c r="X11" t="s">
         <v>241</v>
       </c>
+      <c r="Y11" t="s">
+        <v>409</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB11">
+        <v>30</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>410</v>
+      </c>
+      <c r="AE11">
+        <v>40</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>413</v>
+      </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>139</v>
       </c>
@@ -6636,8 +9574,35 @@
       <c r="X12" t="s">
         <v>38</v>
       </c>
+      <c r="Y12" t="s">
+        <v>416</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB12">
+        <v>21</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>417</v>
+      </c>
+      <c r="AE12">
+        <v>23</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>421</v>
+      </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>148</v>
       </c>
@@ -6710,8 +9675,35 @@
       <c r="X13" t="s">
         <v>38</v>
       </c>
+      <c r="Y13" t="s">
+        <v>424</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB13">
+        <v>9</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>425</v>
+      </c>
+      <c r="AE13">
+        <v>33</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>429</v>
+      </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>157</v>
       </c>
@@ -6784,8 +9776,35 @@
       <c r="X14" t="s">
         <v>38</v>
       </c>
+      <c r="Y14" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB14">
+        <v>18</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>433</v>
+      </c>
+      <c r="AE14">
+        <v>17</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>437</v>
+      </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>168</v>
       </c>
@@ -6858,8 +9877,35 @@
       <c r="X15" t="s">
         <v>304</v>
       </c>
+      <c r="Y15" t="s">
+        <v>440</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB15">
+        <v>12</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>441</v>
+      </c>
+      <c r="AE15">
+        <v>32</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>444</v>
+      </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>176</v>
       </c>
@@ -6932,8 +9978,35 @@
       <c r="X16" t="s">
         <v>311</v>
       </c>
+      <c r="Y16" t="s">
+        <v>447</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB16">
+        <v>25</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>448</v>
+      </c>
+      <c r="AE16">
+        <v>28</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>311</v>
+      </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>184</v>
       </c>
@@ -7006,8 +10079,35 @@
       <c r="X17" t="s">
         <v>38</v>
       </c>
+      <c r="Y17" t="s">
+        <v>452</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>187</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE17">
+        <v>21</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>191</v>
       </c>
@@ -7080,8 +10180,35 @@
       <c r="X18" t="s">
         <v>38</v>
       </c>
+      <c r="Y18" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>187</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE18">
+        <v>8</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>196</v>
       </c>
@@ -7154,8 +10281,35 @@
       <c r="X19" t="s">
         <v>38</v>
       </c>
+      <c r="Y19" t="s">
+        <v>457</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>187</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE19">
+        <v>19</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG19" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>201</v>
       </c>
@@ -7228,8 +10382,35 @@
       <c r="X20" t="s">
         <v>38</v>
       </c>
+      <c r="Y20" t="s">
+        <v>460</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>205</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB20">
+        <v>19</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>461</v>
+      </c>
+      <c r="AE20">
+        <v>23</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>464</v>
+      </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>213</v>
       </c>
@@ -7302,8 +10483,35 @@
       <c r="X21" t="s">
         <v>38</v>
       </c>
+      <c r="Y21" t="s">
+        <v>467</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB21">
+        <v>54</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>187</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>468</v>
+      </c>
+      <c r="AE21">
+        <v>12</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>472</v>
+      </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>218</v>
       </c>
@@ -7376,8 +10584,35 @@
       <c r="X22" t="s">
         <v>38</v>
       </c>
+      <c r="Y22" t="s">
+        <v>475</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB22">
+        <v>57</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>187</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>476</v>
+      </c>
+      <c r="AE22">
+        <v>12</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>480</v>
+      </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>222</v>
       </c>
@@ -7450,8 +10685,35 @@
       <c r="X23" t="s">
         <v>38</v>
       </c>
+      <c r="Y23" t="s">
+        <v>483</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>187</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE23">
+        <v>21</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>227</v>
       </c>
@@ -7524,8 +10786,35 @@
       <c r="X24" t="s">
         <v>38</v>
       </c>
+      <c r="Y24" t="s">
+        <v>486</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB24">
+        <v>33</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>187</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>487</v>
+      </c>
+      <c r="AE24">
+        <v>9</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>491</v>
+      </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>231</v>
       </c>
@@ -7598,9 +10887,36 @@
       <c r="X25" t="s">
         <v>38</v>
       </c>
+      <c r="Y25" t="s">
+        <v>494</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB25">
+        <v>22</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>187</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>495</v>
+      </c>
+      <c r="AE25">
+        <v>3</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG25" t="s">
+        <v>498</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1"/>
+  <autoFilter ref="A1:AG1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Auto-collect traffic data: 2026-10-19 07:42 PM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-10-19_Mon.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-10-19_Mon.xlsx
@@ -7,14 +7,15 @@
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="1_00 PM" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="All Periods Combined" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="7_00 PM" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="All Periods Combined" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2426" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3228" uniqueCount="615">
   <si>
     <t>Date</t>
   </si>
@@ -1519,6 +1520,240 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/1_00_PM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>10/19/2026, 7:04:54 PM</t>
+  </si>
+  <si>
+    <t>7:00 PM</t>
+  </si>
+  <si>
+    <t>Monday (Weekday) - Evening Peak</t>
+  </si>
+  <si>
+    <t> | 56 min | 12.4 km | via Barrackpore Trunk Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:06:35 PM</t>
+  </si>
+  <si>
+    <t> | 1 hr 10 min | 16.3 km | via Netaji Subhas Chandra Bose Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:08:16 PM</t>
+  </si>
+  <si>
+    <t> | 21 min | 4.1 km | via Belgachia Rd/Khudiram Bose Sarani | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:09:57 PM</t>
+  </si>
+  <si>
+    <t> | 29 min | 5.2 km | via Jatindra Mohan Ave and Central Ave/Chittaranjan Ave | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:11:37 PM</t>
+  </si>
+  <si>
+    <t> | 29 min | 5.1 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route, despite crash on Shyama Prasad Mukherjee Rd causing 11-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:11:55 PM</t>
+  </si>
+  <si>
+    <t>Train Walk</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:24 AM—7:42 AM | 32218 - Dankuni - Sealdah Local   | 7:27 AM from Dakshineswar 8 min late |  8 min | Details</t>
+  </si>
+  <si>
+    <t> | 25 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.39x</t>
+  </si>
+  <si>
+    <t>28.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:13:35 PM</t>
+  </si>
+  <si>
+    <t> | 34 min | 8.3 km | via Chowringee Rd/Jawaharlal Nehru Rd and Ashutosh Mukherjee Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:15:18 PM</t>
+  </si>
+  <si>
+    <t> | 32 min | 6.3 km | via Netaji Subhas Chandra Bose Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:16:59 PM</t>
+  </si>
+  <si>
+    <t> | 47 min | 8.8 km | via Jessore Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:18:40 PM</t>
+  </si>
+  <si>
+    <t> | 47 min | 10.8 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:20:20 PM</t>
+  </si>
+  <si>
+    <t> | 27 min | 8.0 km | via Beleghata Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:22:01 PM</t>
+  </si>
+  <si>
+    <t> | 35 min | 7.2 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:23:42 PM</t>
+  </si>
+  <si>
+    <t> | 20 min | 4.9 km | via Narkeldanga Main Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:25:23 PM</t>
+  </si>
+  <si>
+    <t> | 33 min | 7.6 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:27:03 PM</t>
+  </si>
+  <si>
+    <t> | 36 min | 12.7 km | via Mayo Rd and Park St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:28:43 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 9.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:30:25 PM</t>
+  </si>
+  <si>
+    <t> | 10 min | 4.4 km | via Bangaon - Kulpi Rd/Biswa Bangla Sarani/Eastern Metropolitan Bypass/Thakurnagar - Panchpota Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:32:06 PM</t>
+  </si>
+  <si>
+    <t> | 22 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:33:47 PM</t>
+  </si>
+  <si>
+    <t> | 29 min | 7.8 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:35:27 PM</t>
+  </si>
+  <si>
+    <t> | 13 min | 3.7 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:37:08 PM</t>
+  </si>
+  <si>
+    <t> | 16 min | 4.1 km | via NH 12 | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:38:48 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 6.5 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:40:28 PM</t>
+  </si>
+  <si>
+    <t> | 10 min | 2.4 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>10/19/2026, 7:42:09 PM</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-19/7_00_PM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -1598,6 +1833,33 @@
   </si>
   <si>
     <t>1:00 PM Savings (%)</t>
+  </si>
+  <si>
+    <t>7:00 PM Scraped At</t>
+  </si>
+  <si>
+    <t>7:00 PM Actual Metro</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Walk</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Route</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>7:00 PM Car (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Faster Mode</t>
+  </si>
+  <si>
+    <t>7:00 PM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -8387,10 +8649,2124 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:33" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>501</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>12.4</v>
+      </c>
+      <c r="K2" t="s">
+        <v>502</v>
+      </c>
+      <c r="L2" t="s">
+        <v>503</v>
+      </c>
+      <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" t="s">
+        <v>187</v>
+      </c>
+      <c r="P2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2">
+        <v>56</v>
+      </c>
+      <c r="S2" t="s">
+        <v>504</v>
+      </c>
+      <c r="T2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" t="s">
+        <v>38</v>
+      </c>
+      <c r="W2" t="s">
+        <v>38</v>
+      </c>
+      <c r="X2" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>506</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.9</v>
+      </c>
+      <c r="J3">
+        <v>16.3</v>
+      </c>
+      <c r="K3" t="s">
+        <v>502</v>
+      </c>
+      <c r="L3" t="s">
+        <v>503</v>
+      </c>
+      <c r="M3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>38</v>
+      </c>
+      <c r="R3">
+        <v>70</v>
+      </c>
+      <c r="S3" t="s">
+        <v>507</v>
+      </c>
+      <c r="T3" t="s">
+        <v>38</v>
+      </c>
+      <c r="U3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" t="s">
+        <v>38</v>
+      </c>
+      <c r="W3" t="s">
+        <v>38</v>
+      </c>
+      <c r="X3" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>509</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>3.8</v>
+      </c>
+      <c r="J4">
+        <v>4.1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>502</v>
+      </c>
+      <c r="L4" t="s">
+        <v>503</v>
+      </c>
+      <c r="M4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" t="s">
+        <v>187</v>
+      </c>
+      <c r="P4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R4">
+        <v>21</v>
+      </c>
+      <c r="S4" t="s">
+        <v>510</v>
+      </c>
+      <c r="T4" t="s">
+        <v>38</v>
+      </c>
+      <c r="U4" t="s">
+        <v>38</v>
+      </c>
+      <c r="V4" t="s">
+        <v>38</v>
+      </c>
+      <c r="W4" t="s">
+        <v>38</v>
+      </c>
+      <c r="X4" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>5.2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>502</v>
+      </c>
+      <c r="L5" t="s">
+        <v>503</v>
+      </c>
+      <c r="M5" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" t="s">
+        <v>187</v>
+      </c>
+      <c r="P5" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>38</v>
+      </c>
+      <c r="R5">
+        <v>29</v>
+      </c>
+      <c r="S5" t="s">
+        <v>513</v>
+      </c>
+      <c r="T5" t="s">
+        <v>38</v>
+      </c>
+      <c r="U5" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" t="s">
+        <v>38</v>
+      </c>
+      <c r="W5" t="s">
+        <v>38</v>
+      </c>
+      <c r="X5" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>515</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>502</v>
+      </c>
+      <c r="L6" t="s">
+        <v>503</v>
+      </c>
+      <c r="M6" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" t="s">
+        <v>187</v>
+      </c>
+      <c r="P6" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>38</v>
+      </c>
+      <c r="R6">
+        <v>29</v>
+      </c>
+      <c r="S6" t="s">
+        <v>516</v>
+      </c>
+      <c r="T6" t="s">
+        <v>38</v>
+      </c>
+      <c r="U6" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6" t="s">
+        <v>38</v>
+      </c>
+      <c r="W6" t="s">
+        <v>38</v>
+      </c>
+      <c r="X6" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>518</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>6.2</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>502</v>
+      </c>
+      <c r="L7" t="s">
+        <v>503</v>
+      </c>
+      <c r="M7" t="s">
+        <v>38</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>18</v>
+      </c>
+      <c r="P7" t="s">
+        <v>519</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>520</v>
+      </c>
+      <c r="R7">
+        <v>25</v>
+      </c>
+      <c r="S7" t="s">
+        <v>521</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="U7" t="s">
+        <v>522</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>523</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>524</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>526</v>
+      </c>
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>99</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>8.3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>502</v>
+      </c>
+      <c r="L8" t="s">
+        <v>503</v>
+      </c>
+      <c r="M8" t="s">
+        <v>38</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8" t="s">
+        <v>187</v>
+      </c>
+      <c r="P8" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>38</v>
+      </c>
+      <c r="R8">
+        <v>34</v>
+      </c>
+      <c r="S8" t="s">
+        <v>527</v>
+      </c>
+      <c r="T8" t="s">
+        <v>38</v>
+      </c>
+      <c r="U8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V8" t="s">
+        <v>38</v>
+      </c>
+      <c r="W8" t="s">
+        <v>38</v>
+      </c>
+      <c r="X8" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>529</v>
+      </c>
+      <c r="D9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>99</v>
+      </c>
+      <c r="H9" t="s">
+        <v>109</v>
+      </c>
+      <c r="I9">
+        <v>7.1</v>
+      </c>
+      <c r="J9">
+        <v>6.3</v>
+      </c>
+      <c r="K9" t="s">
+        <v>502</v>
+      </c>
+      <c r="L9" t="s">
+        <v>503</v>
+      </c>
+      <c r="M9" t="s">
+        <v>38</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9" t="s">
+        <v>187</v>
+      </c>
+      <c r="P9" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R9">
+        <v>32</v>
+      </c>
+      <c r="S9" t="s">
+        <v>530</v>
+      </c>
+      <c r="T9" t="s">
+        <v>38</v>
+      </c>
+      <c r="U9" t="s">
+        <v>38</v>
+      </c>
+      <c r="V9" t="s">
+        <v>38</v>
+      </c>
+      <c r="W9" t="s">
+        <v>38</v>
+      </c>
+      <c r="X9" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>532</v>
+      </c>
+      <c r="D10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>8.8</v>
+      </c>
+      <c r="J10">
+        <v>8.8</v>
+      </c>
+      <c r="K10" t="s">
+        <v>502</v>
+      </c>
+      <c r="L10" t="s">
+        <v>503</v>
+      </c>
+      <c r="M10" t="s">
+        <v>38</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10" t="s">
+        <v>187</v>
+      </c>
+      <c r="P10" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>38</v>
+      </c>
+      <c r="R10">
+        <v>47</v>
+      </c>
+      <c r="S10" t="s">
+        <v>533</v>
+      </c>
+      <c r="T10" t="s">
+        <v>38</v>
+      </c>
+      <c r="U10" t="s">
+        <v>38</v>
+      </c>
+      <c r="V10" t="s">
+        <v>38</v>
+      </c>
+      <c r="W10" t="s">
+        <v>38</v>
+      </c>
+      <c r="X10" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>535</v>
+      </c>
+      <c r="D11" t="s">
+        <v>127</v>
+      </c>
+      <c r="E11" t="s">
+        <v>128</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" t="s">
+        <v>130</v>
+      </c>
+      <c r="I11">
+        <v>14.2</v>
+      </c>
+      <c r="J11">
+        <v>10.8</v>
+      </c>
+      <c r="K11" t="s">
+        <v>502</v>
+      </c>
+      <c r="L11" t="s">
+        <v>503</v>
+      </c>
+      <c r="M11" t="s">
+        <v>38</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11" t="s">
+        <v>187</v>
+      </c>
+      <c r="P11" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>38</v>
+      </c>
+      <c r="R11">
+        <v>47</v>
+      </c>
+      <c r="S11" t="s">
+        <v>536</v>
+      </c>
+      <c r="T11" t="s">
+        <v>38</v>
+      </c>
+      <c r="U11" t="s">
+        <v>38</v>
+      </c>
+      <c r="V11" t="s">
+        <v>38</v>
+      </c>
+      <c r="W11" t="s">
+        <v>38</v>
+      </c>
+      <c r="X11" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>538</v>
+      </c>
+      <c r="D12" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" t="s">
+        <v>128</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>140</v>
+      </c>
+      <c r="H12" t="s">
+        <v>130</v>
+      </c>
+      <c r="I12">
+        <v>8.6</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>502</v>
+      </c>
+      <c r="L12" t="s">
+        <v>503</v>
+      </c>
+      <c r="M12" t="s">
+        <v>38</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12" t="s">
+        <v>187</v>
+      </c>
+      <c r="P12" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>38</v>
+      </c>
+      <c r="R12">
+        <v>27</v>
+      </c>
+      <c r="S12" t="s">
+        <v>539</v>
+      </c>
+      <c r="T12" t="s">
+        <v>38</v>
+      </c>
+      <c r="U12" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12" t="s">
+        <v>38</v>
+      </c>
+      <c r="W12" t="s">
+        <v>38</v>
+      </c>
+      <c r="X12" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>541</v>
+      </c>
+      <c r="D13" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" t="s">
+        <v>128</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" t="s">
+        <v>140</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>7.2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>502</v>
+      </c>
+      <c r="L13" t="s">
+        <v>503</v>
+      </c>
+      <c r="M13" t="s">
+        <v>38</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13" t="s">
+        <v>187</v>
+      </c>
+      <c r="P13" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>38</v>
+      </c>
+      <c r="R13">
+        <v>35</v>
+      </c>
+      <c r="S13" t="s">
+        <v>542</v>
+      </c>
+      <c r="T13" t="s">
+        <v>38</v>
+      </c>
+      <c r="U13" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13" t="s">
+        <v>38</v>
+      </c>
+      <c r="W13" t="s">
+        <v>38</v>
+      </c>
+      <c r="X13" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>544</v>
+      </c>
+      <c r="D14" t="s">
+        <v>157</v>
+      </c>
+      <c r="E14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>158</v>
+      </c>
+      <c r="H14" t="s">
+        <v>130</v>
+      </c>
+      <c r="I14">
+        <v>6.6</v>
+      </c>
+      <c r="J14">
+        <v>4.9</v>
+      </c>
+      <c r="K14" t="s">
+        <v>502</v>
+      </c>
+      <c r="L14" t="s">
+        <v>503</v>
+      </c>
+      <c r="M14" t="s">
+        <v>38</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14" t="s">
+        <v>187</v>
+      </c>
+      <c r="P14" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>38</v>
+      </c>
+      <c r="R14">
+        <v>20</v>
+      </c>
+      <c r="S14" t="s">
+        <v>545</v>
+      </c>
+      <c r="T14" t="s">
+        <v>38</v>
+      </c>
+      <c r="U14" t="s">
+        <v>38</v>
+      </c>
+      <c r="V14" t="s">
+        <v>38</v>
+      </c>
+      <c r="W14" t="s">
+        <v>38</v>
+      </c>
+      <c r="X14" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>547</v>
+      </c>
+      <c r="D15" t="s">
+        <v>168</v>
+      </c>
+      <c r="E15" t="s">
+        <v>128</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" t="s">
+        <v>158</v>
+      </c>
+      <c r="I15">
+        <v>7.7</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>502</v>
+      </c>
+      <c r="L15" t="s">
+        <v>503</v>
+      </c>
+      <c r="M15" t="s">
+        <v>38</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15" t="s">
+        <v>187</v>
+      </c>
+      <c r="P15" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>38</v>
+      </c>
+      <c r="R15">
+        <v>33</v>
+      </c>
+      <c r="S15" t="s">
+        <v>548</v>
+      </c>
+      <c r="T15" t="s">
+        <v>38</v>
+      </c>
+      <c r="U15" t="s">
+        <v>38</v>
+      </c>
+      <c r="V15" t="s">
+        <v>38</v>
+      </c>
+      <c r="W15" t="s">
+        <v>38</v>
+      </c>
+      <c r="X15" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>550</v>
+      </c>
+      <c r="D16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E16" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>130</v>
+      </c>
+      <c r="I16">
+        <v>11.3</v>
+      </c>
+      <c r="J16">
+        <v>12.7</v>
+      </c>
+      <c r="K16" t="s">
+        <v>502</v>
+      </c>
+      <c r="L16" t="s">
+        <v>503</v>
+      </c>
+      <c r="M16" t="s">
+        <v>38</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16" t="s">
+        <v>187</v>
+      </c>
+      <c r="P16" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>38</v>
+      </c>
+      <c r="R16">
+        <v>36</v>
+      </c>
+      <c r="S16" t="s">
+        <v>551</v>
+      </c>
+      <c r="T16" t="s">
+        <v>38</v>
+      </c>
+      <c r="U16" t="s">
+        <v>38</v>
+      </c>
+      <c r="V16" t="s">
+        <v>38</v>
+      </c>
+      <c r="W16" t="s">
+        <v>38</v>
+      </c>
+      <c r="X16" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>553</v>
+      </c>
+      <c r="D17" t="s">
+        <v>184</v>
+      </c>
+      <c r="E17" t="s">
+        <v>185</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" t="s">
+        <v>186</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>9.8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>502</v>
+      </c>
+      <c r="L17" t="s">
+        <v>503</v>
+      </c>
+      <c r="M17" t="s">
+        <v>38</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17" t="s">
+        <v>187</v>
+      </c>
+      <c r="P17" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17">
+        <v>25</v>
+      </c>
+      <c r="S17" t="s">
+        <v>554</v>
+      </c>
+      <c r="T17" t="s">
+        <v>38</v>
+      </c>
+      <c r="U17" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" t="s">
+        <v>38</v>
+      </c>
+      <c r="W17" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>556</v>
+      </c>
+      <c r="D18" t="s">
+        <v>191</v>
+      </c>
+      <c r="E18" t="s">
+        <v>185</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>192</v>
+      </c>
+      <c r="H18" t="s">
+        <v>186</v>
+      </c>
+      <c r="I18">
+        <v>4.4</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>502</v>
+      </c>
+      <c r="L18" t="s">
+        <v>503</v>
+      </c>
+      <c r="M18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18" t="s">
+        <v>187</v>
+      </c>
+      <c r="P18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R18">
+        <v>10</v>
+      </c>
+      <c r="S18" t="s">
+        <v>557</v>
+      </c>
+      <c r="T18" t="s">
+        <v>38</v>
+      </c>
+      <c r="U18" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" t="s">
+        <v>38</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>559</v>
+      </c>
+      <c r="D19" t="s">
+        <v>196</v>
+      </c>
+      <c r="E19" t="s">
+        <v>185</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>109</v>
+      </c>
+      <c r="H19" t="s">
+        <v>197</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>502</v>
+      </c>
+      <c r="L19" t="s">
+        <v>503</v>
+      </c>
+      <c r="M19" t="s">
+        <v>38</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19" t="s">
+        <v>187</v>
+      </c>
+      <c r="P19" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19">
+        <v>22</v>
+      </c>
+      <c r="S19" t="s">
+        <v>560</v>
+      </c>
+      <c r="T19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U19" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" t="s">
+        <v>38</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>562</v>
+      </c>
+      <c r="D20" t="s">
+        <v>201</v>
+      </c>
+      <c r="E20" t="s">
+        <v>202</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>203</v>
+      </c>
+      <c r="H20" t="s">
+        <v>204</v>
+      </c>
+      <c r="I20">
+        <v>7.9</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>502</v>
+      </c>
+      <c r="L20" t="s">
+        <v>503</v>
+      </c>
+      <c r="M20" t="s">
+        <v>38</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20" t="s">
+        <v>187</v>
+      </c>
+      <c r="P20" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>38</v>
+      </c>
+      <c r="R20">
+        <v>29</v>
+      </c>
+      <c r="S20" t="s">
+        <v>563</v>
+      </c>
+      <c r="T20" t="s">
+        <v>38</v>
+      </c>
+      <c r="U20" t="s">
+        <v>38</v>
+      </c>
+      <c r="V20" t="s">
+        <v>38</v>
+      </c>
+      <c r="W20" t="s">
+        <v>38</v>
+      </c>
+      <c r="X20" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>565</v>
+      </c>
+      <c r="D21" t="s">
+        <v>213</v>
+      </c>
+      <c r="E21" t="s">
+        <v>202</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>214</v>
+      </c>
+      <c r="H21" t="s">
+        <v>204</v>
+      </c>
+      <c r="I21">
+        <v>3.7</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>502</v>
+      </c>
+      <c r="L21" t="s">
+        <v>503</v>
+      </c>
+      <c r="M21" t="s">
+        <v>38</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21" t="s">
+        <v>187</v>
+      </c>
+      <c r="P21" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>38</v>
+      </c>
+      <c r="R21">
+        <v>13</v>
+      </c>
+      <c r="S21" t="s">
+        <v>566</v>
+      </c>
+      <c r="T21" t="s">
+        <v>38</v>
+      </c>
+      <c r="U21" t="s">
+        <v>38</v>
+      </c>
+      <c r="V21" t="s">
+        <v>38</v>
+      </c>
+      <c r="W21" t="s">
+        <v>38</v>
+      </c>
+      <c r="X21" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>568</v>
+      </c>
+      <c r="D22" t="s">
+        <v>218</v>
+      </c>
+      <c r="E22" t="s">
+        <v>202</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>203</v>
+      </c>
+      <c r="H22" t="s">
+        <v>214</v>
+      </c>
+      <c r="I22">
+        <v>4.2</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>502</v>
+      </c>
+      <c r="L22" t="s">
+        <v>503</v>
+      </c>
+      <c r="M22" t="s">
+        <v>38</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22" t="s">
+        <v>187</v>
+      </c>
+      <c r="P22" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>38</v>
+      </c>
+      <c r="R22">
+        <v>16</v>
+      </c>
+      <c r="S22" t="s">
+        <v>569</v>
+      </c>
+      <c r="T22" t="s">
+        <v>38</v>
+      </c>
+      <c r="U22" t="s">
+        <v>38</v>
+      </c>
+      <c r="V22" t="s">
+        <v>38</v>
+      </c>
+      <c r="W22" t="s">
+        <v>38</v>
+      </c>
+      <c r="X22" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>571</v>
+      </c>
+      <c r="D23" t="s">
+        <v>222</v>
+      </c>
+      <c r="E23" t="s">
+        <v>202</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>203</v>
+      </c>
+      <c r="H23" t="s">
+        <v>223</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>502</v>
+      </c>
+      <c r="L23" t="s">
+        <v>503</v>
+      </c>
+      <c r="M23" t="s">
+        <v>38</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23" t="s">
+        <v>187</v>
+      </c>
+      <c r="P23" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>38</v>
+      </c>
+      <c r="R23">
+        <v>25</v>
+      </c>
+      <c r="S23" t="s">
+        <v>572</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" t="s">
+        <v>38</v>
+      </c>
+      <c r="W23" t="s">
+        <v>38</v>
+      </c>
+      <c r="X23" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>574</v>
+      </c>
+      <c r="D24" t="s">
+        <v>227</v>
+      </c>
+      <c r="E24" t="s">
+        <v>202</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>214</v>
+      </c>
+      <c r="H24" t="s">
+        <v>223</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>502</v>
+      </c>
+      <c r="L24" t="s">
+        <v>503</v>
+      </c>
+      <c r="M24" t="s">
+        <v>38</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24" t="s">
+        <v>187</v>
+      </c>
+      <c r="P24" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>38</v>
+      </c>
+      <c r="R24">
+        <v>10</v>
+      </c>
+      <c r="S24" t="s">
+        <v>575</v>
+      </c>
+      <c r="T24" t="s">
+        <v>38</v>
+      </c>
+      <c r="U24" t="s">
+        <v>38</v>
+      </c>
+      <c r="V24" t="s">
+        <v>38</v>
+      </c>
+      <c r="W24" t="s">
+        <v>38</v>
+      </c>
+      <c r="X24" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>577</v>
+      </c>
+      <c r="D25" t="s">
+        <v>231</v>
+      </c>
+      <c r="E25" t="s">
+        <v>202</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>223</v>
+      </c>
+      <c r="H25" t="s">
+        <v>204</v>
+      </c>
+      <c r="I25">
+        <v>1.3</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>502</v>
+      </c>
+      <c r="L25" t="s">
+        <v>503</v>
+      </c>
+      <c r="M25" t="s">
+        <v>38</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25" t="s">
+        <v>187</v>
+      </c>
+      <c r="P25" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>38</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s">
+        <v>232</v>
+      </c>
+      <c r="T25" t="s">
+        <v>38</v>
+      </c>
+      <c r="U25" t="s">
+        <v>38</v>
+      </c>
+      <c r="V25" t="s">
+        <v>38</v>
+      </c>
+      <c r="W25" t="s">
+        <v>38</v>
+      </c>
+      <c r="X25" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>578</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="Y2" r:id="rId1"/>
+    <hyperlink ref="Y3" r:id="rId2"/>
+    <hyperlink ref="Y4" r:id="rId3"/>
+    <hyperlink ref="Y5" r:id="rId4"/>
+    <hyperlink ref="Y6" r:id="rId5"/>
+    <hyperlink ref="X7" r:id="rId6"/>
+    <hyperlink ref="Y7" r:id="rId7"/>
+    <hyperlink ref="Y8" r:id="rId8"/>
+    <hyperlink ref="Y9" r:id="rId9"/>
+    <hyperlink ref="Y10" r:id="rId10"/>
+    <hyperlink ref="Y11" r:id="rId11"/>
+    <hyperlink ref="Y12" r:id="rId12"/>
+    <hyperlink ref="Y13" r:id="rId13"/>
+    <hyperlink ref="Y14" r:id="rId14"/>
+    <hyperlink ref="Y15" r:id="rId15"/>
+    <hyperlink ref="Y16" r:id="rId16"/>
+    <hyperlink ref="Y17" r:id="rId17"/>
+    <hyperlink ref="Y18" r:id="rId18"/>
+    <hyperlink ref="Y19" r:id="rId19"/>
+    <hyperlink ref="Y20" r:id="rId20"/>
+    <hyperlink ref="Y21" r:id="rId21"/>
+    <hyperlink ref="Y22" r:id="rId22"/>
+    <hyperlink ref="Y23" r:id="rId23"/>
+    <hyperlink ref="Y24" r:id="rId24"/>
+    <hyperlink ref="Y25" r:id="rId25"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AP25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:42" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -8410,88 +10786,115 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>501</v>
+        <v>579</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>502</v>
+        <v>580</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>503</v>
+        <v>581</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>504</v>
+        <v>582</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>505</v>
+        <v>583</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>506</v>
+        <v>584</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>507</v>
+        <v>585</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>508</v>
+        <v>586</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>509</v>
+        <v>587</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>510</v>
+        <v>588</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>511</v>
+        <v>589</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>512</v>
+        <v>590</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>513</v>
+        <v>591</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>514</v>
+        <v>592</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>515</v>
+        <v>593</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>516</v>
+        <v>594</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>517</v>
+        <v>595</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>518</v>
+        <v>596</v>
       </c>
       <c r="Y1" s="4" t="s">
-        <v>519</v>
+        <v>597</v>
       </c>
       <c r="Z1" s="4" t="s">
-        <v>520</v>
+        <v>598</v>
       </c>
       <c r="AA1" s="4" t="s">
-        <v>521</v>
+        <v>599</v>
       </c>
       <c r="AB1" s="4" t="s">
-        <v>522</v>
+        <v>600</v>
       </c>
       <c r="AC1" s="4" t="s">
-        <v>523</v>
+        <v>601</v>
       </c>
       <c r="AD1" s="4" t="s">
-        <v>524</v>
+        <v>602</v>
       </c>
       <c r="AE1" s="4" t="s">
-        <v>525</v>
+        <v>603</v>
       </c>
       <c r="AF1" s="4" t="s">
-        <v>526</v>
+        <v>604</v>
       </c>
       <c r="AG1" s="4" t="s">
-        <v>527</v>
+        <v>605</v>
+      </c>
+      <c r="AH1" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="AI1" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="AJ1" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="AK1" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="AL1" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="AM1" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="AN1" s="4" t="s">
+        <v>612</v>
+      </c>
+      <c r="AO1" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="AP1" s="4" t="s">
+        <v>614</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -8591,8 +10994,35 @@
       <c r="AG2" t="s">
         <v>348</v>
       </c>
+      <c r="AH2" t="s">
+        <v>501</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN2">
+        <v>56</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -8692,8 +11122,35 @@
       <c r="AG3" t="s">
         <v>356</v>
       </c>
+      <c r="AH3" t="s">
+        <v>506</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN3">
+        <v>70</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -8793,8 +11250,35 @@
       <c r="AG4" t="s">
         <v>364</v>
       </c>
+      <c r="AH4" t="s">
+        <v>509</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN4">
+        <v>21</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -8894,8 +11378,35 @@
       <c r="AG5" t="s">
         <v>372</v>
       </c>
+      <c r="AH5" t="s">
+        <v>512</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN5">
+        <v>29</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -8995,8 +11506,35 @@
       <c r="AG6" t="s">
         <v>86</v>
       </c>
+      <c r="AH6" t="s">
+        <v>515</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN6">
+        <v>29</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -9096,8 +11634,35 @@
       <c r="AG7" t="s">
         <v>384</v>
       </c>
+      <c r="AH7" t="s">
+        <v>518</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK7">
+        <v>18</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>519</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>520</v>
+      </c>
+      <c r="AN7">
+        <v>25</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>523</v>
+      </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>98</v>
       </c>
@@ -9197,8 +11762,35 @@
       <c r="AG8" t="s">
         <v>391</v>
       </c>
+      <c r="AH8" t="s">
+        <v>526</v>
+      </c>
+      <c r="AI8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN8">
+        <v>34</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>108</v>
       </c>
@@ -9298,8 +11890,35 @@
       <c r="AG9" t="s">
         <v>398</v>
       </c>
+      <c r="AH9" t="s">
+        <v>529</v>
+      </c>
+      <c r="AI9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK9" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN9">
+        <v>32</v>
+      </c>
+      <c r="AO9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -9399,8 +12018,35 @@
       <c r="AG10" t="s">
         <v>406</v>
       </c>
+      <c r="AH10" t="s">
+        <v>532</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN10">
+        <v>47</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>127</v>
       </c>
@@ -9500,8 +12146,35 @@
       <c r="AG11" t="s">
         <v>413</v>
       </c>
+      <c r="AH11" t="s">
+        <v>535</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK11" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN11">
+        <v>47</v>
+      </c>
+      <c r="AO11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP11" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>139</v>
       </c>
@@ -9601,8 +12274,35 @@
       <c r="AG12" t="s">
         <v>421</v>
       </c>
+      <c r="AH12" t="s">
+        <v>538</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK12" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN12">
+        <v>27</v>
+      </c>
+      <c r="AO12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP12" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>148</v>
       </c>
@@ -9702,8 +12402,35 @@
       <c r="AG13" t="s">
         <v>429</v>
       </c>
+      <c r="AH13" t="s">
+        <v>541</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK13" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN13">
+        <v>35</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP13" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>157</v>
       </c>
@@ -9803,8 +12530,35 @@
       <c r="AG14" t="s">
         <v>437</v>
       </c>
+      <c r="AH14" t="s">
+        <v>544</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK14" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN14">
+        <v>20</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP14" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>168</v>
       </c>
@@ -9904,8 +12658,35 @@
       <c r="AG15" t="s">
         <v>444</v>
       </c>
+      <c r="AH15" t="s">
+        <v>547</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN15">
+        <v>33</v>
+      </c>
+      <c r="AO15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP15" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>176</v>
       </c>
@@ -10005,8 +12786,35 @@
       <c r="AG16" t="s">
         <v>311</v>
       </c>
+      <c r="AH16" t="s">
+        <v>550</v>
+      </c>
+      <c r="AI16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN16">
+        <v>36</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP16" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>184</v>
       </c>
@@ -10106,8 +12914,35 @@
       <c r="AG17" t="s">
         <v>38</v>
       </c>
+      <c r="AH17" t="s">
+        <v>553</v>
+      </c>
+      <c r="AI17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN17">
+        <v>25</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP17" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>191</v>
       </c>
@@ -10207,8 +13042,35 @@
       <c r="AG18" t="s">
         <v>38</v>
       </c>
+      <c r="AH18" t="s">
+        <v>556</v>
+      </c>
+      <c r="AI18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK18" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN18">
+        <v>10</v>
+      </c>
+      <c r="AO18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP18" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>196</v>
       </c>
@@ -10308,8 +13170,35 @@
       <c r="AG19" t="s">
         <v>38</v>
       </c>
+      <c r="AH19" t="s">
+        <v>559</v>
+      </c>
+      <c r="AI19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN19">
+        <v>22</v>
+      </c>
+      <c r="AO19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP19" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>201</v>
       </c>
@@ -10409,8 +13298,35 @@
       <c r="AG20" t="s">
         <v>464</v>
       </c>
+      <c r="AH20" t="s">
+        <v>562</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN20">
+        <v>29</v>
+      </c>
+      <c r="AO20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP20" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>213</v>
       </c>
@@ -10510,8 +13426,35 @@
       <c r="AG21" t="s">
         <v>472</v>
       </c>
+      <c r="AH21" t="s">
+        <v>565</v>
+      </c>
+      <c r="AI21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN21">
+        <v>13</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP21" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>218</v>
       </c>
@@ -10611,8 +13554,35 @@
       <c r="AG22" t="s">
         <v>480</v>
       </c>
+      <c r="AH22" t="s">
+        <v>568</v>
+      </c>
+      <c r="AI22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK22" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN22">
+        <v>16</v>
+      </c>
+      <c r="AO22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP22" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>222</v>
       </c>
@@ -10712,8 +13682,35 @@
       <c r="AG23" t="s">
         <v>38</v>
       </c>
+      <c r="AH23" t="s">
+        <v>571</v>
+      </c>
+      <c r="AI23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK23" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN23">
+        <v>25</v>
+      </c>
+      <c r="AO23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP23" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>227</v>
       </c>
@@ -10813,8 +13810,35 @@
       <c r="AG24" t="s">
         <v>491</v>
       </c>
+      <c r="AH24" t="s">
+        <v>574</v>
+      </c>
+      <c r="AI24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN24">
+        <v>10</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP24" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>231</v>
       </c>
@@ -10914,9 +13938,36 @@
       <c r="AG25" t="s">
         <v>498</v>
       </c>
+      <c r="AH25" t="s">
+        <v>577</v>
+      </c>
+      <c r="AI25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK25" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN25">
+        <v>3</v>
+      </c>
+      <c r="AO25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP25" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG1"/>
+  <autoFilter ref="A1:AP1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>